<commit_message>
Update tracker: number ranges done, launchpad-hosted UI decision recorded
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -757,7 +757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1023,22 +1023,22 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Shared docNo generation per company or group-global; needed before any document module</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Configurable per object: scope GLOBAL or COMPANY, and pattern, set independently</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
+          <t>GLOBAL issues RR-2026-0001/RES-2026-0001; COMPANY issues BUD-INFC-2026-0001 and BUD-PMI-2026-0001 advancing independently; numbers issued on draft activation, not draft creation</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Build next, before Masters</t>
         </is>
       </c>
     </row>
@@ -1711,59 +1711,59 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>U-04</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Launchpad intents declared</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rates, vendors; scoped GROUP/COMPANY + promotion queue</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
+          <t>manifest parses; two inbounds registered</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>Start after P-06</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>U-05</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Launchpad-hosted shell (blend with S/4)</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
+          <t>App must render inside the Fiori launchpad shell; its own sap.tnt.ToolPage chrome duplicates launchpad header, search, user menu and side nav</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -1778,29 +1778,29 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>After Masters</t>
+          <t>Strip app shell to content only</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>U-06</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Spaces and Pages navigation</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+          <t>S/4 Public Cloud style. Launchpad CONFIGURATION (CDM site / Work Zone), not CDS entities</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -1810,56 +1810,56 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>sandbox2 confirmed present in the local 1.150.0 runtime, so this is reproducible locally</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>Build FLP sandbox site</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>U-07</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Morning Horizon theme</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -1869,12 +1869,12 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>Resource hierarchy, CBS library, rates, vendors; scoped GROUP/COMPANY + promotion queue</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -1889,14 +1889,14 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>Start after P-06</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -1906,12 +1906,12 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -1926,14 +1926,14 @@
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -1943,12 +1943,12 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -1963,14 +1963,14 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -1980,12 +1980,12 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -2000,14 +2000,14 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2017,12 +2017,12 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -2037,66 +2037,66 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>mta.yaml completion</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>No approuter module, no UI module</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>At risk</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>db-deployer path corrected to db/</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Fix before first CF deploy</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -2111,42 +2111,190 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
+          <t>B-08</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Project Commercial</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Client billing, variations, payment certificates</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>After Execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>B-09</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Plant Department</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Last per your sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>mta.yaml completion</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>No approuter module, no UI module</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>db-deployer path corrected to db/</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Fix before first CF deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C45" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D45" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="E45" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="G45" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -2167,7 +2315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2669,6 +2817,117 @@
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>D-13</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Number range scope is configurable per object, not a product-wide choice</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Your instruction. Scope (GLOBAL/COMPANY) and pattern are configured independently so a client can print the company code while running one group series, or vice versa</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Low — configuration only</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>D-14</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Document numbers are issued on draft activation, not draft creation</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Abandoned drafts would otherwise burn numbers and leave gaps in the series</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Claude (technical)</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Low, but gap-free numbering is sometimes an audit requirement — confirm if so</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>D-15</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>UI is launchpad-hosted; Spaces and Pages are launchpad configuration, not application data</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Your requirement to blend with S/4HANA. The shell, theme and navigation come from the launchpad; the app renders content only. Modelling spaces as CDS entities was started and abandoned as wrong for this target</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>High — supersedes part of D-05; the app's own ToolPage shell must be removed</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
@@ -2689,7 +2948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2760,59 +3019,59 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Document number ranges: per company (RR-INFC-2026-0001) or group-global (RR-2026-0001)?</t>
+          <t>Document number ranges: per company or group-global?</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Every document module depends on it; changing later means renumbering live data</t>
+          <t>ANSWERED: configurable per object. Built and verified both scopes</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Per company / group-global / configurable per object type</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>P-06, then all of Masters onward</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Before Masters</t>
+          <t>Answered 2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Q-02</t>
+          <t>Q-13</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>What is in the EC&amp;O starter content pack?</t>
+          <t>Where does KONSTRYX surface for the end user — SAP Build Work Zone, or the S/4HANA Public Cloud launchpad directly?</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>You chose 'code lists ship, starter pack as optional import'. I need to know what the pack contains before building the import</t>
+          <t>Decides how Spaces and Pages are configured and how our apps federate with standard S/4 content. Work Zone is the usual route for BTP apps alongside S/4</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy depth, CBS library, productivity/consumption norms, trade catalogue</t>
+          <t>SAP Build Work Zone (federates S/4 content) / S/4 launchpad content manager / both</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>B-01 Masters, B-02 Templates</t>
+          <t>U-05, U-06, D-01 mta.yaml</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
@@ -2822,34 +3081,34 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Before Masters</t>
+          <t>Before first CF deploy</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Q-03</t>
+          <t>Q-14</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Approval schemes: who approves what, at which value bands?</t>
+          <t>Does numbering need to be gap-free for audit?</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>The framework is built but has no content. Needs real thresholds per object per company</t>
+          <t>Numbers are issued on activation so abandoned drafts do not consume them, but a cancelled document still leaves a gap. Some jurisdictions require unbroken sequences for certain document types</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Per object type: steps, approver persona, amount bands</t>
+          <t>Gaps acceptable (current) / gap-free required for named document types</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>F-02 Approval engine</t>
+          <t>P-06</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
@@ -2866,27 +3125,27 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Q-04</t>
+          <t>Q-02</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Attachment storage: SAP Object Store or HANA LOB?</t>
+          <t>What is in the EC&amp;O starter content pack?</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Object Store needs a CF service instance and changes the upload path; HANA LOB is simpler but costlier at volume</t>
+          <t>You chose 'code lists ship, starter pack as optional import'. I need to know what the pack contains before building the import</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Object Store (recommended for drawings/photos) / HANA LOB</t>
+          <t>Resource hierarchy depth, CBS library, productivity/consumption norms, trade catalogue</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>F-04</t>
+          <t>B-01 Masters, B-02 Templates</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
@@ -2896,34 +3155,34 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Before Uploads</t>
+          <t>Before Masters</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Q-05</t>
+          <t>Q-03</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>The canonical demo numbers do not reconcile</t>
+          <t>Approval schemes: who approves what, at which value bands?</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Wireframe header says AED 716,044; the five line values sum to 685,080 and match the per-WBS commitment split exactly. L1 rate 320/day implies 115,200 not 276,480</t>
+          <t>The framework is built but has no content. Needs real thresholds per object per company</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Correct the header to 685,080 / correct L1 rate to 768 / supply the intended figures</t>
+          <t>Per object type: steps, approver persona, amount bands</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Any stakeholder demo</t>
+          <t>F-02 Approval engine</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -2933,34 +3192,34 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Before first demo</t>
+          <t>Before Budgeting</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Q-06</t>
+          <t>Q-04</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>BOQ import template — confirm the column set</t>
+          <t>Attachment storage: SAP Object Store or HANA LOB?</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Named the highest-risk item in your own requirements register. The importer is built to the template, not the reverse</t>
+          <t>Object Store needs a CF service instance and changes the upload path; HANA LOB is simpler but costlier at volume</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Provide the actual client BOQ template(s) you must accept</t>
+          <t>Object Store (recommended for drawings/photos) / HANA LOB</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>B-04 Uploads</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
@@ -2977,27 +3236,27 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Q-07</t>
+          <t>Q-05</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>CBS instance versioning: copy-on-create or live reference to the library?</t>
+          <t>The canonical demo numbers do not reconcile</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Open item in Data Model Spec section 10. Affects whether library changes propagate into running projects</t>
+          <t>Wireframe header says AED 716,044; the five line values sum to 685,080 and match the per-WBS commitment split exactly. L1 rate 320/day implies 115,200 not 276,480</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Copy-on-create (proposed) / live reference</t>
+          <t>Correct the header to 685,080 / correct L1 rate to 768 / supply the intended figures</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>B-01, B-03</t>
+          <t>Any stakeholder demo</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -3007,34 +3266,34 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Before Project Setup</t>
+          <t>Before first demo</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Q-08</t>
+          <t>Q-06</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Encumbrance currency: company currency or group reporting currency?</t>
+          <t>BOQ import template — confirm the column set</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Open item in Data Model Spec section 10</t>
+          <t>Named the highest-risk item in your own requirements register. The importer is built to the template, not the reverse</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Company ccy + group conversion in ins (proposed) / group ccy</t>
+          <t>Provide the actual client BOQ template(s) you must accept</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>B-06 Budgeting</t>
+          <t>B-04 Uploads</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
@@ -3044,34 +3303,34 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Before Budgeting</t>
+          <t>Before Uploads</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Q-09</t>
+          <t>Q-07</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud dev tenant access</t>
+          <t>CBS instance versioning: copy-on-create or live reference to the library?</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>No connector can be built or validated without it. Named as a prerequisite in the phase plan</t>
+          <t>Open item in Data Model Spec section 10. Affects whether library changes propagate into running projects</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Provide tenant + communication arrangements</t>
+          <t>Copy-on-create (proposed) / live reference</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>B-01, B-03</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
@@ -3088,27 +3347,27 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Q-10</t>
+          <t>Q-08</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Scope re-baseline: personalization + attachments + approvals on every screen</t>
+          <t>Encumbrance currency: company currency or group reporting currency?</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Wireframe v12 is 41 modules / 434 screens. The 22-week MVP plan with 1 UI5 developer does not carry this</t>
+          <t>Open item in Data Model Spec section 10</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Re-baseline the plan / reduce MVP screen scope / add UI capacity</t>
+          <t>Company ccy + group conversion in ins (proposed) / group ccy</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Overall plan credibility</t>
+          <t>B-06 Budgeting</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -3118,34 +3377,34 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Before committing a client date</t>
+          <t>Before Budgeting</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Q-11</t>
+          <t>Q-09</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>UI5 production delivery: how is the app served in Cloud Foundry?</t>
+          <t>S/4HANA Public Cloud dev tenant access</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>mta.yaml has no approuter and no UI module today, and the app bootstraps from a local runtime path</t>
+          <t>No connector can be built or validated without it. Named as a prerequisite in the phase plan</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Approuter + HTML5 repo (standard) / other</t>
+          <t>Provide tenant + communication arrangements</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>D-02</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -3155,42 +3414,116 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Before first CF deploy</t>
+          <t>Before Project Setup</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
+          <t>Q-10</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Scope re-baseline: personalization + attachments + approvals on every screen</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Wireframe v12 is 41 modules / 434 screens. The 22-week MVP plan with 1 UI5 developer does not carry this</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Re-baseline the plan / reduce MVP screen scope / add UI capacity</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Overall plan credibility</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Before committing a client date</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Q-11</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>UI5 production delivery: how is the app served in Cloud Foundry?</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>mta.yaml has no approuter and no UI module today, and the app bootstraps from a local runtime path</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Approuter + HTML5 repo (standard) / other</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Before first CF deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
           <t>Q-12</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>CI/CD tooling</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Prerequisite 4 in the phase plan, still undecided</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>SAP CI/CD service / GitHub Actions / Azure DevOps</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>Before team scales up</t>
         </is>
@@ -3211,7 +3544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3309,7 +3642,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Shared docNo generation service</t>
+          <t>Configurable scope (GLOBAL/COMPANY) and pattern per object; issued on activation</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -3319,37 +3652,39 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Q-01</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Q-01 (answered)</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
-        <v>3</v>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>2b</t>
+        </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Launchpad-hosted shell</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rates, vendors, scoped GROUP/COMPANY + promotion queue</t>
+          <t>Strip the app's own ToolPage chrome; FLP sandbox with Spaces and Pages for local dev</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Your sequence. Everything downstream references master codes</t>
+          <t>Blend with S/4HANA. Doing this before the screen count grows avoids stripping the shell out of every screen later</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Q-01, Q-02</t>
+          <t>Q-13</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -3360,26 +3695,26 @@
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
+          <t>Resource hierarchy, CBS library, rates, vendors, scoped GROUP/COMPANY + promotion queue</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Your sequence. Templates are composed of masters</t>
+          <t>Your sequence. Everything downstream references master codes</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Q-01, Q-02</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -3390,26 +3725,26 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance, S/4 Enterprise Project mirror</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Your sequence. Instantiates a template</t>
+          <t>Your sequence. Templates are composed of masters</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Templates, Q-07, Q-09</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -3420,26 +3755,26 @@
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>Project, WBS, CBS instance, S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Your sequence. Needs a project to import into. Highest-risk item in the plan</t>
+          <t>Your sequence. Instantiates a template</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Project Setup, Q-04, Q-06</t>
+          <t>Templates, Q-07, Q-09</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -3450,26 +3785,26 @@
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Your sequence. Activities hang off WBS</t>
+          <t>Your sequence. Needs a project to import into. Highest-risk item in the plan</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Project Setup, Q-04, Q-06</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -3480,26 +3815,26 @@
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Your sequence. Needs BOQ and CBS to exist</t>
+          <t>Your sequence. Activities hang off WBS</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Uploads, Q-03, Q-08</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -3510,26 +3845,26 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower, chain steps 5-10</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Your sequence. Consumes budget; encumbrance must exist first</t>
+          <t>Your sequence. Needs BOQ and CBS to exist</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Uploads, Q-03, Q-08</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -3540,26 +3875,26 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower, chain steps 5-10</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Your sequence. Bills against executed work</t>
+          <t>Your sequence. Consumes budget; encumbrance must exist first</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Execution</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -3570,29 +3905,59 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Project Commercial</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Client billing, variations, payment certificates</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Your sequence. Bills against executed work</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Plant Department</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Equipment, fleet, scaffolding/formwork</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Your sequence — explicitly after the core</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Execution</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
Log upgrade-safety issue: db/data resets client configuration on redeploy
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -3978,7 +3978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4596,6 +4596,43 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>I-16</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Upgrade safety</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Client configuration in db/data is reset on every upgrade</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>cds build --production generates konstryx.nr-NumberRangeObject.hdbtabledata. HDI re-imports managed rows on redeploy, so a client who changes a number range scope or pattern would silently have it reverted at the next upgrade. NumberRangeObjects is writable in the service, so this is reachable</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Move client-configurable rows out of db/data into the one-time onboarding import; keep db/data for immutable delivered catalogue only (Activity, Module, AuthObject, Currencies - all @readonly)</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
Update tracker: Option A recorded, shell removed, two issues logged
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1772,22 +1772,22 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>App must render inside the Fiori launchpad shell; its own sap.tnt.ToolPage chrome duplicates launchpad header, search, user menu and side nav</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
+          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>Strip app shell to content only</t>
         </is>
       </c>
     </row>
@@ -1809,29 +1809,29 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>S/4 Public Cloud style. Launchpad CONFIGURATION (CDM site / Work Zone), not CDS entities</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>sandbox2 confirmed present in the local 1.150.0 runtime, so this is reproducible locally</t>
+          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Build FLP sandbox site</t>
+          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>U-07</t>
+          <t>U-08</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -1841,71 +1841,71 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Morning Horizon theme</t>
+          <t>Split into task-focused apps per document type</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
+          <t>Register more intents as screens are built</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>U-07</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Morning Horizon theme</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rates, vendors; scoped GROUP/COMPANY + promotion queue</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Start after P-06</t>
+          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -1915,12 +1915,12 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
+          <t>Resource hierarchy, CBS library, rates, vendors; scoped GROUP/COMPANY + promotion queue</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -1935,14 +1935,14 @@
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>After Masters</t>
+          <t>Start after P-06</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -1952,12 +1952,12 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -1972,14 +1972,14 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -1989,12 +1989,12 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -2009,14 +2009,14 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2026,12 +2026,12 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -2046,14 +2046,14 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2063,12 +2063,12 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -2083,14 +2083,14 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2100,12 +2100,12 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -2120,14 +2120,14 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2137,12 +2137,12 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -2157,14 +2157,14 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Client billing, variations, payment certificates</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -2194,51 +2194,51 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>mta.yaml completion</t>
+          <t>Plant Department</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>No approuter module, no UI module</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>At risk</t>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>db-deployer path corrected to db/</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Fix before first CF deploy</t>
+          <t>Last per your sequence</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>D-01</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2248,62 +2248,99 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>mta.yaml completion</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>No approuter module, no UI module</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>db-deployer path corrected to db/</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>Fix before first CF deploy</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D46" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -4750,7 +4787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5371,35 +5408,109 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
+          <t>I-17</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Authorization</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Enforcement broke every worklist request with HTTP 500</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>The handler filters on catalogue paths project.code and company.code, but RequestOverview is a grouped projection that exposed projectCode as a flat string and dropped both associations. Missed because enforcement was verified against the service directly and the UI was not re-tested after</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>View now exposes the project and company associations. Worth adding a startup check that every declared path resolves on every projection, so this fails at boot rather than per request</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>I-18</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Local FLP sandbox does not boot</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>flp.html fails with 'Cannot read properties of null (reading src)'. sandbox2 is deprecated since 1.136 and the newer sap/ushell/sandbox boot contract differs</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Open — either finish the sandbox boot or verify launchpad integration directly on BTP</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
           <t>I-16</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Upgrade safety</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Client configuration in db/data is reset on every upgrade</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>cds build --production generates konstryx.nr-NumberRangeObject.hdbtabledata. HDI re-imports managed rows on redeploy, so a client who changes a number range scope or pattern would silently have it reverted at the next upgrade. NumberRangeObjects is writable in the service, so this is reachable</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Move client-configurable rows out of db/data into the one-time onboarding import; keep db/data for immutable delivered catalogue only (Activity, Module, AuthObject, Currencies - all @readonly)</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Update tracker: I-16 closed, content pack mechanism recorded
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1017,7 +1017,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>P-06</t>
+          <t>P-07</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1027,12 +1027,12 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Document number ranges</t>
+          <t>Delivered content pack mechanism</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Configurable per object: scope GLOBAL or COMPANY, and pattern, set independently</t>
+          <t>Versioned packs applied insert-if-missing, in version order; ships in the jar and readable from ./content; applyContentPacks admin action for upgrades without restart</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -1042,34 +1042,34 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>GLOBAL issues RR-2026-0001/RES-2026-0001; COMPANY issues BUD-INFC-2026-0001 and BUD-PMI-2026-0001 advancing independently; numbers issued on draft activation, not draft creation</t>
+          <t>Client edit survived an upgrade pack that contained the same row: 1 inserted, 1 left untouched, client scope preserved</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Reuse for the EC&amp;O starter pack (Q-02)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>A-01</t>
+          <t>P-06</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Authorization model (S/4 style)</t>
+          <t>Document number ranges</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>AuthObject + Activity + Persona + PersonaPermission + UserAssignment scoped by company/project</t>
+          <t>Configurable per object: scope GLOBAL or COMPANY, and pattern, set independently</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Catalogue: 7 modules, 21 objects, 6 activities</t>
+          <t>GLOBAL issues RR-2026-0001/RES-2026-0001; COMPANY issues BUD-INFC-2026-0001 and BUD-PMI-2026-0001 advancing independently; numbers issued on draft activation, not draft creation</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1091,7 +1091,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>A-02</t>
+          <t>A-01</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>EffectivePermission view</t>
+          <t>Authorization model (S/4 style)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Flattens assignments x grants to answer 'what can this person do'</t>
+          <t>AuthObject + Activity + Persona + PersonaPermission + UserAssignment scoped by company/project</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>23 rows resolved for the 4 seeded personas</t>
+          <t>Catalogue: 7 modules, 21 objects, 6 activities</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1128,7 +1128,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>A-03</t>
+          <t>A-02</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -1138,12 +1138,12 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Runtime enforcement handler</t>
+          <t>EffectivePermission view</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Activity check + company/project instance filtering on every CRUD event</t>
+          <t>Flattens assignments x grants to answer 'what can this person do'</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Scoped user sees 4 of 5 requests; unrestricted sees 5; own $filter still ANDs; no grant = 403</t>
+          <t>23 rows resolved for the 4 seeded personas</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1165,7 +1165,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>A-04</t>
+          <t>A-03</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -1175,34 +1175,34 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Write-path input-data check</t>
+          <t>Runtime enforcement handler</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Reject CREATE/UPDATE carrying a project outside the user's scope</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Activity check + company/project instance filtering on every CRUD event</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
+          <t>Scoped user sees 4 of 5 requests; unrestricted sees 5; own $filter still ANDs; no grant = 403</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Validate after Project Setup exists</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>A-05</t>
+          <t>A-04</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -1212,12 +1212,12 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Administration UI</t>
+          <t>Write-path input-data check</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>S/4-like screens to maintain personas, grants, assignments</t>
+          <t>Reject CREATE/UPDATE carrying a project outside the user's scope</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -1232,51 +1232,51 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Part of Masters/Admin UI block</t>
+          <t>Validate after Project Setup exists</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>F-01</t>
+          <t>A-05</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Approval framework model</t>
+          <t>Administration UI</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Schemes per object type, ordered steps, approver persona, value bands, runtime instances</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>S/4-like screens to maintain personas, grants, assignments</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Engine not built</t>
+          <t>Part of Masters/Admin UI block</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>F-02</t>
+          <t>F-01</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -1286,34 +1286,34 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Approval engine</t>
+          <t>Approval framework model</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Instantiate on submit, match value bands, advance steps, audit</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Schemes per object type, ordered steps, approver persona, value bands, runtime instances</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting model</t>
+          <t>Engine not built</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>F-03</t>
+          <t>F-02</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1323,34 +1323,34 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Attachments model</t>
+          <t>Approval engine</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Polymorphic on entityName+objectID, media-type content, categories</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Instantiate on submit, match value bands, advance steps, audit</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Upload handler + object store not built</t>
+          <t>After Budgeting model</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>F-04</t>
+          <t>F-03</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -1360,34 +1360,34 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Attachment upload + storage</t>
+          <t>Attachments model</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Object store binding for Cloud Foundry vs HANA LOB</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Polymorphic on entityName+objectID, media-type content, categories</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Decision needed (see Open Decisions)</t>
+          <t>Upload handler + object store not built</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>F-05</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1397,34 +1397,34 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Table personalization store</t>
+          <t>Attachment upload + storage</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>UserVariant entity holding UI5 p13n state per user</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Object store binding for Cloud Foundry vs HANA LOB</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Not wired to any table yet</t>
+          <t>Decision needed (see Open Decisions)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>F-06</t>
+          <t>F-05</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1434,71 +1434,71 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Table personalization UI wiring</t>
+          <t>Table personalization store</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>p13n + VariantManagement on every list screen</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>UserVariant entity holding UI5 p13n state per user</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Apply as each screen is built</t>
+          <t>Not wired to any table yet</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>M-01</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Workflow spine RR-&gt;ADV-&gt;AVC-&gt;RES</t>
+          <t>Table personalization UI wiring</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Vertical-agnostic, multi-line, seeded with canonical EQR thread</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>p13n + VariantManagement on every list screen</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Queryable over OData; 5 lines, AED 685,080</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Apply as each screen is built</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>M-02</t>
+          <t>M-01</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1508,12 +1508,12 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>WBS on request line</t>
+          <t>Workflow spine RR-&gt;ADV-&gt;AVC-&gt;RES</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Spec section 6 requires one WBS per line; was missing</t>
+          <t>Vertical-agnostic, multi-line, seeded with canonical EQR thread</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>3 distinct WBS across the 5 EQR lines</t>
+          <t>Queryable over OData; 5 lines, AED 685,080</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1535,7 +1535,7 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>M-03</t>
+          <t>M-02</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1545,12 +1545,12 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>EQR vertical extension</t>
+          <t>WBS on request line</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Instances, mob/demob window, own-vs-rental, vendor, operators</t>
+          <t>Spec section 6 requires one WBS per line; was missing</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>$expand=equipment,wbs returns all 5 lines resolved</t>
+          <t>3 distinct WBS across the 5 EQR lines</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1572,7 +1572,7 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>M-04</t>
+          <t>M-03</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1582,71 +1582,71 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Chain steps CMT/MOB/OPL/VAR/DMB/CLS</t>
+          <t>EQR vertical extension</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Steps 5-10 have no CDS entities at all</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Instances, mob/demob window, own-vs-rental, vendor, operators</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
+          <t>$expand=equipment,wbs returns all 5 lines resolved</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>Part of Project Execution block</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>U-01</t>
+          <t>M-04</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>RR worklist on live OData</t>
+          <t>Chain steps CMT/MOB/OPL/VAR/DMB/CLS</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>RequestOverview projection, server-side filters</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Steps 5-10 have no CDS entities at all</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Verified in browser: 4 requests, EQR shows 5 lines / 685,080; EQR filter issues new $batch</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Part of Project Execution block</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>U-02</t>
+          <t>U-01</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1656,34 +1656,34 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Request detail page on OData</t>
+          <t>RR worklist on live OData</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Still reads webapp/model/data.json</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>RequestOverview projection, server-side filters</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
+          <t>Verified in browser: 4 requests, EQR shows 5 lines / 685,080; EQR filter issues new $batch</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
-        <is>
-          <t>Now unblocked by M-03</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>U-03</t>
+          <t>U-02</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1693,17 +1693,17 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Chain step pages on OData</t>
+          <t>Request detail page on OData</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Still read data.json</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Still reads webapp/model/data.json</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -1713,14 +1713,14 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Blocked by M-04</t>
+          <t>Now unblocked by M-03</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>U-04</t>
+          <t>U-03</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1730,34 +1730,34 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Launchpad intents declared</t>
+          <t>Chain step pages on OData</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Still read data.json</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>manifest parses; two inbounds registered</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Blocked by M-04</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>U-05</t>
+          <t>U-04</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1767,12 +1767,12 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Launchpad-hosted shell (blend with S/4)</t>
+          <t>Launchpad intents declared</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
+          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
+          <t>manifest parses; two inbounds registered</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1794,7 +1794,7 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>U-06</t>
+          <t>U-05</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -1804,34 +1804,34 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Spaces and Pages navigation</t>
+          <t>Launchpad-hosted shell (blend with S/4)</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>At risk</t>
+          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
+          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>U-08</t>
+          <t>U-06</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -1841,34 +1841,34 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Split into task-focused apps per document type</t>
+          <t>Spaces and Pages navigation</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Register more intents as screens are built</t>
+          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>U-07</t>
+          <t>U-08</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -1878,71 +1878,71 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Morning Horizon theme</t>
+          <t>Split into task-focused apps per document type</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
+          <t>Register more intents as screens are built</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>U-07</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Morning Horizon theme</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rates, vendors; scoped GROUP/COMPANY + promotion queue</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Start after P-06</t>
+          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-01</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -1952,12 +1952,12 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
+          <t>Resource hierarchy, CBS library, rates, vendors; scoped GROUP/COMPANY + promotion queue</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -1972,14 +1972,14 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>After Masters</t>
+          <t>Start after P-06</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -1989,12 +1989,12 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -2009,14 +2009,14 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2026,12 +2026,12 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -2046,14 +2046,14 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2063,12 +2063,12 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -2083,14 +2083,14 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2100,12 +2100,12 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -2120,14 +2120,14 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2137,12 +2137,12 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -2157,14 +2157,14 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -2194,14 +2194,14 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2211,12 +2211,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Client billing, variations, payment certificates</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -2231,51 +2231,51 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>mta.yaml completion</t>
+          <t>Plant Department</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>No approuter module, no UI module</t>
-        </is>
-      </c>
-      <c r="E44" s="9" t="inlineStr">
-        <is>
-          <t>At risk</t>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>db-deployer path corrected to db/</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Fix before first CF deploy</t>
+          <t>Last per your sequence</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>D-01</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2285,62 +2285,99 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>mta.yaml completion</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>No approuter module, no UI module</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>db-deployer path corrected to db/</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>Fix before first CF deploy</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C47" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D47" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -4787,7 +4824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5497,20 +5534,94 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>cds build --production generates konstryx.nr-NumberRangeObject.hdbtabledata. HDI re-imports managed rows on redeploy, so a client who changes a number range scope or pattern would silently have it reverted at the next upgrade. NumberRangeObjects is writable in the service, so this is reachable</t>
+          <t>cds build --production generates konstryx.nr-NumberRangeObject.hdbtabledata. HDI re-imports managed rows on redeploy, so a client who changes a number range scope or pattern would silently have it reverted at the next upgrade</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Move client-configurable rows out of db/data into the one-time onboarding import; keep db/data for immutable delivered catalogue only (Activity, Module, AuthObject, Currencies - all @readonly)</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Fixed: configurable content moved to versioned packs applied insert-if-missing. Proven — client re-scoped RR to COMPANY, an upgrade pack containing an RR row was applied, RR kept the client's scope and only the new row arrived</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>I-19</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Content packs</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Packs applied in filename order, not version order</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>number-ranges-v2.json sorted before number-ranges.json because '-' precedes '.', so 1.0.1 applied before 1.0.0 and the base pack reported its own rows as pre-existing</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Sort by packId then zero-padded version segments, so 1.0.10 follows 1.0.9</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>I-20</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Number ranges</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>A range configured on an entity without docNo would fail every create</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>konstryx.wf.AdvisoryDecision has no document number; the handler would have written the field regardless</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Handler now skips targets with no docNo element, so a misconfiguration is ignored rather than breaking creates</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Update tracker: Masters scope and promotion queue done
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1942,7 +1942,7 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>B-01</t>
+          <t>B-01a</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -1952,34 +1952,34 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Masters — hybrid scope enforcement</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rates, vendors; scoped GROUP/COMPANY + promotion queue</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
+          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>Start after P-06</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-01b</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -1989,34 +1989,34 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Masters — promotion queue (mdg)</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
+          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-01c</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2026,12 +2026,12 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Masters — validation rules</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+          <t>Hierarchy integrity (L5 parent must be L4), code uniqueness within scope, rate effective-dating overlaps</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -2046,14 +2046,14 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>Next</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-01d</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2063,12 +2063,12 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Masters — remaining entities + UI</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>CBS library, productivity and consumption norms, templates under the same scope treatment; Masters screens</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -2083,14 +2083,14 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>After validation</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2100,12 +2100,12 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -2120,14 +2120,14 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2137,12 +2137,12 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -2157,14 +2157,14 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -2194,14 +2194,14 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2211,12 +2211,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -2231,14 +2231,14 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -2268,66 +2268,66 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>mta.yaml completion</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>No approuter module, no UI module</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="inlineStr">
-        <is>
-          <t>At risk</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>db-deployer path corrected to db/</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Fix before first CF deploy</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
+          <t>Client billing, variations, payment certificates</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -2342,42 +2342,153 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
+          <t>B-09</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Plant Department</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Last per your sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>mta.yaml completion</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>No approuter module, no UI module</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>db-deployer path corrected to db/</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Fix before first CF deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -4824,7 +4935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5593,35 +5704,109 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
+          <t>I-21</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Company-scoped authorization hid every group-scoped master</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>I-22</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Promotion approval threw NullPointerException</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Use a HashMap for update payloads that clear fields</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
           <t>I-20</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Number ranges</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>A range configured on an entity without docNo would fail every create</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>konstryx.wf.AdvisoryDecision has no document number; the handler would have written the field regardless</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>Handler now skips targets with no docNo element, so a misconfiguration is ignored rather than breaking creates</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Update tracker: Masters validation done, composition defect logged
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -2031,22 +2031,22 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Hierarchy integrity (L5 parent must be L4), code uniqueness within scope, rate effective-dating overlaps</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
+          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>Next</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5704,27 +5704,27 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>I-21</t>
+          <t>I-23</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Company-scoped authorization hid every group-scoped master</t>
+          <t>Self-referencing compositions crashed draft activation</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
+          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
+          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
@@ -5741,7 +5741,7 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>I-22</t>
+          <t>I-21</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -5751,17 +5751,17 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Promotion approval threw NullPointerException</t>
+          <t>Company-scoped authorization hid every group-scoped master</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Use a HashMap for update payloads that clear fields</t>
+          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -5778,35 +5778,72 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
+          <t>I-22</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Promotion approval threw NullPointerException</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Use a HashMap for update payloads that clear fields</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
           <t>I-20</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>Number ranges</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>A range configured on an entity without docNo would fail every create</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>konstryx.wf.AdvisoryDecision has no document number; the handler would have written the field regardless</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>Handler now skips targets with no docNo element, so a misconfiguration is ignored rather than breaking creates</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Update tracker: MTA now builds; deployment blocked on a BTP target
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2433,34 +2433,34 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>mta.yaml completion</t>
+          <t>MTA builds a deployable archive</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>No approuter module, no UI module</t>
-        </is>
-      </c>
-      <c r="E49" s="9" t="inlineStr">
-        <is>
-          <t>At risk</t>
+          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>db-deployer path corrected to db/</t>
+          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Fix before first CF deploy</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>D-04</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2470,17 +2470,17 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>First Cloud Foundry deployment</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
@@ -2490,42 +2490,79 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B52" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E52" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
+      <c r="F52" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -4972,7 +5009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5455,22 +5492,22 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>mta.yaml has no approuter module and no UI module</t>
+          <t>mta.yaml had no approuter, so nothing a browser could reach</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Cannot deploy to Cloud Foundry at all yet</t>
+          <t>The project had never produced a deployable archive</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Approuter added with XSUAA login and token forwarding; mbt build now produces konstryx_0.1.0.mtar (68.9 MB) with the exec jar, router, 234 HDI artifacts and xs-security.json</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -5482,27 +5519,27 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>I-13</t>
+          <t>I-24</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Demo data</t>
+          <t>Deployment</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Wireframe request header (716,044) does not reconcile with its own line values (685,080)</t>
+          <t>No BTP target available for KONSTRYX</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Any stakeholder demo shows inconsistent totals</t>
+          <t>The CF CLI is targeted at an unrelated client subaccount (LAND MARK INTERNATIONAL) and its token has expired. The archive is built but cannot be pushed</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Needs a KONSTRYX subaccount with Cloud Foundry, HANA Cloud and XSUAA entitlements, and a fresh cf login</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -5519,22 +5556,22 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>I-14</t>
+          <t>I-13</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Plan</t>
+          <t>Demo data</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Personalization, attachments and approvals on every object were not in the 22-week MVP estimate</t>
+          <t>Wireframe request header (716,044) does not reconcile with its own line values (685,080)</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Plan credibility; 434 screens each inherit this layer</t>
+          <t>Any stakeholder demo shows inconsistent totals</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -5556,27 +5593,27 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>I-15</t>
+          <t>I-14</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Plan</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Admin persona cannot read workflow/project services</t>
+          <t>Personalization, attachments and approvals on every object were not in the 22-week MVP estimate</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Service-level @requires still gates entry by XSUAA role; the Admin mock user lacks those roles</t>
+          <t>Plan credibility; 434 screens each inherit this layer</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>By design today, but role collections need reviewing before go-live</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
@@ -5593,7 +5630,7 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>I-17</t>
+          <t>I-15</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -5603,22 +5640,22 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Enforcement broke every worklist request with HTTP 500</t>
+          <t>Admin persona cannot read workflow/project services</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>The handler filters on catalogue paths project.code and company.code, but RequestOverview is a grouped projection that exposed projectCode as a flat string and dropped both associations. Missed because enforcement was verified against the service directly and the UI was not re-tested after</t>
+          <t>Service-level @requires still gates entry by XSUAA role; the Admin mock user lacks those roles</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>View now exposes the project and company associations. Worth adding a startup check that every declared path resolves on every projection, so this fails at boot rather than per request</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>Closed</t>
+          <t>By design today, but role collections need reviewing before go-live</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -5630,32 +5667,32 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>I-18</t>
+          <t>I-17</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Local FLP sandbox does not boot</t>
+          <t>Enforcement broke every worklist request with HTTP 500</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>flp.html fails with 'Cannot read properties of null (reading src)'. sandbox2 is deprecated since 1.136 and the newer sap/ushell/sandbox boot contract differs</t>
+          <t>The handler filters on catalogue paths project.code and company.code, but RequestOverview is a grouped projection that exposed projectCode as a flat string and dropped both associations. Missed because enforcement was verified against the service directly and the UI was not re-tested after</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Open — either finish the sandbox boot or verify launchpad integration directly on BTP</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>View now exposes the project and company associations. Worth adding a startup check that every declared path resolves on every projection, so this fails at boot rather than per request</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -5667,32 +5704,32 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>I-16</t>
+          <t>I-18</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Upgrade safety</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Client configuration in db/data is reset on every upgrade</t>
+          <t>Local FLP sandbox does not boot</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>cds build --production generates konstryx.nr-NumberRangeObject.hdbtabledata. HDI re-imports managed rows on redeploy, so a client who changes a number range scope or pattern would silently have it reverted at the next upgrade</t>
+          <t>flp.html fails with 'Cannot read properties of null (reading src)'. sandbox2 is deprecated since 1.136 and the newer sap/ushell/sandbox boot contract differs</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Fixed: configurable content moved to versioned packs applied insert-if-missing. Proven — client re-scoped RR to COMPANY, an upgrade pack containing an RR row was applied, RR kept the client's scope and only the new row arrived</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Closed</t>
+          <t>Open — either finish the sandbox boot or verify launchpad integration directly on BTP</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -5704,27 +5741,27 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>I-19</t>
+          <t>I-16</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Content packs</t>
+          <t>Upgrade safety</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Packs applied in filename order, not version order</t>
+          <t>Client configuration in db/data is reset on every upgrade</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>number-ranges-v2.json sorted before number-ranges.json because '-' precedes '.', so 1.0.1 applied before 1.0.0 and the base pack reported its own rows as pre-existing</t>
+          <t>cds build --production generates konstryx.nr-NumberRangeObject.hdbtabledata. HDI re-imports managed rows on redeploy, so a client who changes a number range scope or pattern would silently have it reverted at the next upgrade</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Sort by packId then zero-padded version segments, so 1.0.10 follows 1.0.9</t>
+          <t>Fixed: configurable content moved to versioned packs applied insert-if-missing. Proven — client re-scoped RR to COMPANY, an upgrade pack containing an RR row was applied, RR kept the client's scope and only the new row arrived</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
@@ -5741,27 +5778,27 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>I-23</t>
+          <t>I-19</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Content packs</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Self-referencing compositions crashed draft activation</t>
+          <t>Packs applied in filename order, not version order</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
+          <t>number-ranges-v2.json sorted before number-ranges.json because '-' precedes '.', so 1.0.1 applied before 1.0.0 and the base pack reported its own rows as pre-existing</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
+          <t>Sort by packId then zero-padded version segments, so 1.0.10 follows 1.0.9</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
@@ -5778,27 +5815,27 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>I-21</t>
+          <t>I-23</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Company-scoped authorization hid every group-scoped master</t>
+          <t>Self-referencing compositions crashed draft activation</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
+          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
+          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -5815,7 +5852,7 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>I-22</t>
+          <t>I-21</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -5825,17 +5862,17 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Promotion approval threw NullPointerException</t>
+          <t>Company-scoped authorization hid every group-scoped master</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Use a HashMap for update payloads that clear fields</t>
+          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
@@ -5852,35 +5889,72 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
+          <t>I-22</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Promotion approval threw NullPointerException</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Use a HashMap for update payloads that clear fields</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
           <t>I-20</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Number ranges</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>A range configured on an entity without docNo would fail every create</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>konstryx.wf.AdvisoryDecision has no document number; the handler would have written the field regardless</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>Handler now skips targets with no docNo element, so a misconfiguration is ignored rather than breaking creates</t>
         </is>
       </c>
-      <c r="F28" s="10" t="inlineStr">
+      <c r="F29" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Update tracker: Masters list screens done, blank-screen and cds-dk issues logged
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2100,34 +2100,34 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Masters — screens</t>
+          <t>Masters — list screens</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>List and object pages for resource hierarchy, CBS library, rates and norms, plus the promotion queue</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
+          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>Next; needs the launchpad shell decision already taken (D-16)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-01f</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2137,12 +2137,12 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Masters — object pages</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
+          <t>Drill into a single master to view and edit; the pattern every later module reuses</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -2157,14 +2157,14 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>After Masters</t>
+          <t>Next in Masters</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-01g</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Masters — productivity and consumption norms</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+          <t>Screens plus seed data; norms drive derived consumption and earned value</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -2194,14 +2194,14 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>After object pages</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2211,12 +2211,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -2231,14 +2231,14 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -2268,14 +2268,14 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2285,12 +2285,12 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -2305,14 +2305,14 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2322,12 +2322,12 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -2342,14 +2342,14 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2359,12 +2359,12 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -2379,14 +2379,14 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2396,12 +2396,12 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -2416,71 +2416,71 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>MTA builds a deployable archive</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Client billing, variations, payment certificates</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>First Cloud Foundry deployment</t>
+          <t>Plant Department</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
-        </is>
-      </c>
-      <c r="E50" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
@@ -2490,14 +2490,14 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+          <t>Last per your sequence</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>D-01</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2507,62 +2507,136 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>MTA builds a deployable archive</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
+          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>Needs S/4 dev tenant access</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>First Cloud Foundry deployment</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr">
+      <c r="E54" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G54" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -5009,7 +5083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5815,27 +5889,27 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>I-23</t>
+          <t>I-25</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Self-referencing compositions crashed draft activation</t>
+          <t>Blank screen after the app shell was removed</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
+          <t>Stripping sap.tnt.ToolPage removed the control establishing layout height. UI5 injects a UIArea div that takes no height of its own, and the NavContainer below sets overflow:hidden - so every control was clipped to nothing while still reporting a correct size. DOM text, network and per-element geometry checks all passed while the screen was empty</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
+          <t>Declared the full height chain in style.css. Found by painting a test div (which showed) and then walking the ancestor chain to #container-uiarea</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -5852,27 +5926,27 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>I-21</t>
+          <t>I-26</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Company-scoped authorization hid every group-scoped master</t>
+          <t>mbt build silently removes cds-dk</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
+          <t>The MTA build runs npm install --production at the root, pruning devDependencies. @sap/cds-dk goes with them and the next Maven build fails with 'cds' is not recognized</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
+          <t>Run npm install after an MTA build</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
@@ -5889,27 +5963,27 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>I-22</t>
+          <t>I-23</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Promotion approval threw NullPointerException</t>
+          <t>Self-referencing compositions crashed draft activation</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Use a HashMap for update payloads that clear fields</t>
+          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
@@ -5926,35 +6000,109 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
+          <t>I-21</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Company-scoped authorization hid every group-scoped master</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>I-22</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Promotion approval threw NullPointerException</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Use a HashMap for update payloads that clear fields</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>I-20</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Number ranges</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>A range configured on an entity without docNo would fail every create</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>konstryx.wf.AdvisoryDecision has no document number; the handler would have written the field regardless</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>Handler now skips targets with no docNo element, so a misconfiguration is ignored rather than breaking creates</t>
         </is>
       </c>
-      <c r="F29" s="10" t="inlineStr">
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Tracker: add Suggestions sheet; record draft editing and hierarchy fixes
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2149,34 +2149,34 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Masters — object pages</t>
+          <t>Masters — object page</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Drill into a single master to view and edit; the pattern every later module reuses</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
+          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>Next in Masters</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>B-01g</t>
+          <t>B-01h</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2186,34 +2186,34 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Masters — productivity and consumption norms</t>
+          <t>Masters — draft editing</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Screens plus seed data; norms drive derived consumption and earned value</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>After object pages</t>
+          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-01g</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Masters — productivity and consumption norms</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
+          <t>Screens plus seed data; norms drive derived consumption and earned value</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -2243,14 +2243,14 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>After Masters</t>
+          <t>After object pages</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2260,12 +2260,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -2280,14 +2280,14 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2297,12 +2297,12 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -2317,14 +2317,14 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2334,12 +2334,12 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -2354,14 +2354,14 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2371,12 +2371,12 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -2391,14 +2391,14 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2408,12 +2408,12 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -2428,14 +2428,14 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2445,12 +2445,12 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -2465,14 +2465,14 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2482,12 +2482,12 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Client billing, variations, payment certificates</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -2502,51 +2502,51 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>MTA builds a deployable archive</t>
+          <t>Plant Department</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Last per your sequence</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>D-01</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2556,34 +2556,34 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>First Cloud Foundry deployment</t>
+          <t>MTA builds a deployable archive</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
-        </is>
-      </c>
-      <c r="E52" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
+          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>D-04</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2593,17 +2593,17 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>First Cloud Foundry deployment</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
@@ -2613,42 +2613,79 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="D55" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E54" s="7" t="inlineStr">
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
+      <c r="F55" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G55" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -5728,7 +5765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6534,27 +6571,27 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>I-25</t>
+          <t>I-27</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Test data</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Blank screen after the app shell was removed</t>
+          <t>Seed data violated the model's own hierarchy rule</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Stripping sap.tnt.ToolPage removed the control establishing layout height. UI5 injects a UIArea div that takes no height of its own, and the NavContainer below sets overflow:hidden - so every control was clipped to nothing while still reporting a correct size. DOM text, network and per-element geometry checks all passed while the screen was empty</t>
+          <t>Every resource was an L5 with no parent, so activation failed with 'L5 needs a parent at L4' and no seeded master could be edited or saved. 'Below this node' was empty on every page</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Declared the full height chain in style.css. Found by painting a test div (which showed) and then walking the ancestor chain to #container-uiarea</t>
+          <t>Replaced with a real L1-L5 tree of 28 nodes, leaf IDs preserved so rates and request lines still resolve</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -6571,27 +6608,27 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>I-26</t>
+          <t>I-28</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>mbt build silently removes cds-dk</t>
+          <t>Draft editing failed three ways</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>The MTA build runs npm install --production at the root, pruning devDependencies. @sap/cds-dk goes with them and the next Maven build fails with 'cds' is not recognized</t>
+          <t>draftActivate bound against the draftEdit operation context produced nested deferred bindings; expanding associations on a draft failed with 'invalid segment' and swallowed the edit-mode switch; draftEdit refused a second draft, making a master permanently uneditable after a mid-edit tab close</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Run npm install after an MTA build</t>
+          <t>Re-resolve the draft as an ordinary context, expand only the stored record, and resume an existing draft rather than erroring</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
@@ -6608,27 +6645,27 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>I-23</t>
+          <t>I-25</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Self-referencing compositions crashed draft activation</t>
+          <t>Blank screen after the app shell was removed</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
+          <t>Stripping sap.tnt.ToolPage removed the control establishing layout height. UI5 injects a UIArea div that takes no height of its own, and the NavContainer below sets overflow:hidden - so every control was clipped to nothing while still reporting a correct size. DOM text, network and per-element geometry checks all passed while the screen was empty</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
+          <t>Declared the full height chain in style.css. Found by painting a test div (which showed) and then walking the ancestor chain to #container-uiarea</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
@@ -6645,27 +6682,27 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>I-21</t>
+          <t>I-26</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Company-scoped authorization hid every group-scoped master</t>
+          <t>mbt build silently removes cds-dk</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
+          <t>The MTA build runs npm install --production at the root, pruning devDependencies. @sap/cds-dk goes with them and the next Maven build fails with 'cds' is not recognized</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
+          <t>Run npm install after an MTA build</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
@@ -6682,27 +6719,27 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>I-22</t>
+          <t>I-23</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Promotion approval threw NullPointerException</t>
+          <t>Self-referencing compositions crashed draft activation</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Use a HashMap for update payloads that clear fields</t>
+          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
@@ -6719,35 +6756,109 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
+          <t>I-21</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Company-scoped authorization hid every group-scoped master</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>I-22</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Promotion approval threw NullPointerException</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Use a HashMap for update payloads that clear fields</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
           <t>I-20</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Number ranges</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>A range configured on an entity without docNo would fail every create</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>konstryx.wf.AdvisoryDecision has no document number; the handler would have written the field regardless</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
         <is>
           <t>Handler now skips targets with no docNo element, so a misconfiguration is ignored rather than breaking creates</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F33" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Tracker: template instantiation done, ProjectService association gap logged
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2260,34 +2260,34 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Templates — model and instantiation</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree plus default resources, instantiated at project setup</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
+          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>Next block in your sequence</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-02b</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2297,12 +2297,12 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Templates — screen</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
+          <t>List and object page; instantiate action from the UI rather than the API</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -2317,14 +2317,14 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>After Masters</t>
+          <t>Next</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2334,12 +2334,12 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -2354,14 +2354,14 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2371,12 +2371,12 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -2391,14 +2391,14 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2408,12 +2408,12 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -2428,14 +2428,14 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2445,12 +2445,12 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -2465,14 +2465,14 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2482,12 +2482,12 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -2502,14 +2502,14 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2519,12 +2519,12 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2556,12 +2556,12 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Client billing, variations, payment certificates</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -2576,51 +2576,51 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>MTA builds a deployable archive</t>
+          <t>Plant Department</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Last per your sequence</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>D-01</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2630,34 +2630,34 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>First Cloud Foundry deployment</t>
+          <t>MTA builds a deployable archive</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
+          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>D-04</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2667,17 +2667,17 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>First Cloud Foundry deployment</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -2687,42 +2687,79 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="D57" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E56" s="7" t="inlineStr">
+      <c r="E57" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F57" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G57" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -5802,7 +5839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6608,27 +6645,27 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>I-27</t>
+          <t>I-29</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Test data</t>
+          <t>Services</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Seed data violated the model's own hierarchy rule</t>
+          <t>ProjectService dropped associations to master data</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Every resource was an L5 with no parent, so activation failed with 'L5 needs a parent at L4' and no seeded master could be edited or saved. 'Below this node' was empty on every page</t>
+          <t>CAP omits an association whose target is not exposed in the same service, so a project CBS node could not say which library node it came from and a planned resource could not name its resource. ProjectResources was unusable in a UI</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Replaced with a real L1-L5 tree of 28 nodes, leaf IDs preserved so rates and request lines still resolve</t>
+          <t>Expose ResourceCatalog and CBSLibrary read-only in ProjectService for resolution; maintenance stays in MasterDataService</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -6645,27 +6682,27 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>I-28</t>
+          <t>I-27</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Test data</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Draft editing failed three ways</t>
+          <t>Seed data violated the model's own hierarchy rule</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>draftActivate bound against the draftEdit operation context produced nested deferred bindings; expanding associations on a draft failed with 'invalid segment' and swallowed the edit-mode switch; draftEdit refused a second draft, making a master permanently uneditable after a mid-edit tab close</t>
+          <t>Every resource was an L5 with no parent, so activation failed with 'L5 needs a parent at L4' and no seeded master could be edited or saved. 'Below this node' was empty on every page</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Re-resolve the draft as an ordinary context, expand only the stored record, and resume an existing draft rather than erroring</t>
+          <t>Replaced with a real L1-L5 tree of 28 nodes, leaf IDs preserved so rates and request lines still resolve</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
@@ -6682,7 +6719,7 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>I-25</t>
+          <t>I-28</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -6692,17 +6729,17 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Blank screen after the app shell was removed</t>
+          <t>Draft editing failed three ways</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Stripping sap.tnt.ToolPage removed the control establishing layout height. UI5 injects a UIArea div that takes no height of its own, and the NavContainer below sets overflow:hidden - so every control was clipped to nothing while still reporting a correct size. DOM text, network and per-element geometry checks all passed while the screen was empty</t>
+          <t>draftActivate bound against the draftEdit operation context produced nested deferred bindings; expanding associations on a draft failed with 'invalid segment' and swallowed the edit-mode switch; draftEdit refused a second draft, making a master permanently uneditable after a mid-edit tab close</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Declared the full height chain in style.css. Found by painting a test div (which showed) and then walking the ancestor chain to #container-uiarea</t>
+          <t>Re-resolve the draft as an ordinary context, expand only the stored record, and resume an existing draft rather than erroring</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
@@ -6719,27 +6756,27 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>I-26</t>
+          <t>I-25</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>mbt build silently removes cds-dk</t>
+          <t>Blank screen after the app shell was removed</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>The MTA build runs npm install --production at the root, pruning devDependencies. @sap/cds-dk goes with them and the next Maven build fails with 'cds' is not recognized</t>
+          <t>Stripping sap.tnt.ToolPage removed the control establishing layout height. UI5 injects a UIArea div that takes no height of its own, and the NavContainer below sets overflow:hidden - so every control was clipped to nothing while still reporting a correct size. DOM text, network and per-element geometry checks all passed while the screen was empty</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Run npm install after an MTA build</t>
+          <t>Declared the full height chain in style.css. Found by painting a test div (which showed) and then walking the ancestor chain to #container-uiarea</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
@@ -6756,27 +6793,27 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>I-23</t>
+          <t>I-26</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Self-referencing compositions crashed draft activation</t>
+          <t>mbt build silently removes cds-dk</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
+          <t>The MTA build runs npm install --production at the root, pruning devDependencies. @sap/cds-dk goes with them and the next Maven build fails with 'cds' is not recognized</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
+          <t>Run npm install after an MTA build</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
@@ -6793,27 +6830,27 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>I-21</t>
+          <t>I-23</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Masters</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Company-scoped authorization hid every group-scoped master</t>
+          <t>Self-referencing compositions crashed draft activation</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
+          <t>ResourceNode, CBSNode and CBSInstance each declared children as a Composition of themselves. CAP expands compositions recursively on draft activation, so activating any hierarchy master died with a stack overflow in DraftActionsHandler. Composition also implies cascade-delete, so removing an L2 would have taken its subtree with it</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
+          <t>Changed to Association to many; the hierarchy is owned by parent and children are the inverse</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
@@ -6830,7 +6867,7 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>I-22</t>
+          <t>I-21</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -6840,17 +6877,17 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Promotion approval threw NullPointerException</t>
+          <t>Company-scoped authorization hid every group-scoped master</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+          <t>Scoped masters declared companyPath in the authorization catalogue, so the handler added owningCompany.code = 'INFC', which is null on every GROUP row. Each steward saw only their own local master and none of the five shared ones</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Use a HashMap for update payloads that clear fields</t>
+          <t>The company dimension for scoped entities now belongs to MasterScopeHandler alone; the catalogue declares no companyPath for them</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
@@ -6867,35 +6904,72 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
+          <t>I-22</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Masters</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Promotion approval threw NullPointerException</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Map.of rejects null values and clearing owningCompany_ID is precisely a null</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Use a HashMap for update payloads that clear fields</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
           <t>I-20</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>Number ranges</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>A range configured on an entity without docNo would fail every create</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>konstryx.wf.AdvisoryDecision has no document number; the handler would have written the field regardless</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>Handler now skips targets with no docNo element, so a misconfiguration is ignored rather than breaking creates</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr">
+      <c r="F34" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Tracker: approval engine done, five new flags, three closed issues
Records what the approval work decided and what it left open. The flags
worth your attention are S-19 (the delivered value bands are figures I
invented, not your policy) and S-21 (nothing withdraws an approval when the
document it approved is later edited).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>git, 9 commits</t>
+          <t>git, 48 commits</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Engine not built</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1340,29 +1340,29 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Instantiate on submit, match value bands, advance steps, audit</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Instantiate on submit, match value bands, advance steps, enforce approver persona and separation of duties, delegate, withdraw, audit</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>28 checks against the running service: bands select 1/2/3 steps at 50k/300k/2m; out-of-order, double, reasonless and same-person decisions all refused; persona configured through the admin API then enforced</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting model</t>
+          <t>Inbox screen (F-04) and per-object wiring (F-05)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>F-03</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -1372,34 +1372,34 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Attachments model</t>
+          <t>Approval inbox screen</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Polymorphic on entityName+objectID, media-type content, categories</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>The steps awaiting the signed-in user, with approve, reject and delegate</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Upload handler + object store not built</t>
+          <t>With the UI rebuild</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>F-04</t>
+          <t>F-05</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Attachment upload + storage</t>
+          <t>Wire submit into each object's lifecycle</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Object store binding for Cloud Foundry vs HANA LOB</t>
+          <t>Today the caller chooses when to submit. Each document type should move to 'In Approval' on submit and act on the outcome</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -1429,14 +1429,14 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Decision needed (see Open Decisions)</t>
+          <t>Per module as each is built</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>F-05</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1446,12 +1446,12 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Table personalization store</t>
+          <t>Content pack references</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>UserVariant entity holding UI5 p13n state per user</t>
+          <t>Packs can name another row instead of its UUID, and match on composite natural keys; each pack applies atomically</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1461,19 +1461,19 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>APPROVAL_SCHEMES resolves auth objects and its own schemes at deploy time: 6 rows inserted</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Not wired to any table yet</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>F-06</t>
+          <t>F-03</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1483,86 +1483,86 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Table personalization UI wiring</t>
+          <t>Attachments model</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>p13n + VariantManagement on every list screen</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Polymorphic on entityName+objectID, media-type content, categories</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Apply as each screen is built</t>
+          <t>Upload handler + object store not built</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>M-01</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Workflow spine RR-&gt;ADV-&gt;AVC-&gt;RES</t>
+          <t>Attachment upload + storage</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Vertical-agnostic, multi-line, seeded with canonical EQR thread</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Object store binding for Cloud Foundry vs HANA LOB</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Queryable over OData; 5 lines, AED 685,080</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Decision needed (see Open Decisions)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>M-02</t>
+          <t>F-05</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>WBS on request line</t>
+          <t>Table personalization store</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Spec section 6 requires one WBS per line; was missing</t>
+          <t>UserVariant entity holding UI5 p13n state per user</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1572,56 +1572,56 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>3 distinct WBS across the 5 EQR lines</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Not wired to any table yet</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>M-03</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>EQR vertical extension</t>
+          <t>Table personalization UI wiring</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Instances, mob/demob window, own-vs-rental, vendor, operators</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>p13n + VariantManagement on every list screen</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>$expand=equipment,wbs returns all 5 lines resolved</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Apply as each screen is built</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>M-04</t>
+          <t>M-01</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1631,49 +1631,49 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Chain steps CMT/MOB/OPL/VAR/DMB/CLS</t>
+          <t>Workflow spine RR-&gt;ADV-&gt;AVC-&gt;RES</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Steps 5-10 have no CDS entities at all</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Vertical-agnostic, multi-line, seeded with canonical EQR thread</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
+          <t>Queryable over OData; 5 lines, AED 685,080</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>Part of Project Execution block</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>U-01</t>
+          <t>M-02</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>RR worklist on live OData</t>
+          <t>WBS on request line</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>RequestOverview projection, server-side filters</t>
+          <t>Spec section 6 requires one WBS per line; was missing</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Verified in browser: 4 requests, EQR shows 5 lines / 685,080; EQR filter issues new $batch</t>
+          <t>3 distinct WBS across the 5 EQR lines</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1695,64 +1695,64 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>U-02</t>
+          <t>M-03</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Request detail page on OData</t>
+          <t>EQR vertical extension</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Still reads webapp/model/data.json</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Instances, mob/demob window, own-vs-rental, vendor, operators</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
+          <t>$expand=equipment,wbs returns all 5 lines resolved</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>Now unblocked by M-03</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>U-03</t>
+          <t>M-04</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Chain step pages on OData</t>
+          <t>Chain steps CMT/MOB/OPL/VAR/DMB/CLS</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Still read data.json</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Steps 5-10 have no CDS entities at all</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -1762,14 +1762,14 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Blocked by M-04</t>
+          <t>Part of Project Execution block</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>U-04</t>
+          <t>U-01</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -1779,12 +1779,12 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Launchpad intents declared</t>
+          <t>RR worklist on live OData</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
+          <t>RequestOverview projection, server-side filters</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>manifest parses; two inbounds registered</t>
+          <t>Verified in browser: 4 requests, EQR shows 5 lines / 685,080; EQR filter issues new $batch</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1806,7 +1806,7 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>U-05</t>
+          <t>U-02</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -1816,34 +1816,34 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Launchpad-hosted shell (blend with S/4)</t>
+          <t>Request detail page on OData</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Still reads webapp/model/data.json</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Now unblocked by M-03</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>U-06</t>
+          <t>U-03</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -1853,34 +1853,34 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Spaces and Pages navigation</t>
+          <t>Chain step pages on OData</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
+          <t>Still read data.json</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
+          <t>Blocked by M-04</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>U-08</t>
+          <t>U-04</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -1890,34 +1890,34 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Split into task-focused apps per document type</t>
+          <t>Launchpad intents declared</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
+          <t>manifest parses; two inbounds registered</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
-        <is>
-          <t>Register more intents as screens are built</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>U-07</t>
+          <t>U-05</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -1927,12 +1927,12 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Morning Horizon theme</t>
+          <t>Launchpad-hosted shell (blend with S/4)</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
+          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -1942,108 +1942,108 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
+          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>B-01a</t>
+          <t>U-06</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Masters — hybrid scope enforcement</t>
+          <t>Spaces and Pages navigation</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
+          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>B-01b</t>
+          <t>U-08</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Masters — promotion queue (mdg)</t>
+          <t>Split into task-focused apps per document type</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Register more intents as screens are built</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>B-01c</t>
+          <t>U-07</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Masters — validation rules</t>
+          <t>Morning Horizon theme</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
+          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -2053,19 +2053,19 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
+          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>B-01d</t>
+          <t>B-01a</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -2075,12 +2075,12 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Masters — remaining entities catalogued</t>
+          <t>Masters — hybrid scope enforcement</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>CBS library, productivity and consumption norms, templates, material mirror added to the authorization catalogue</t>
+          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>CBS library picked up isolation, promotion and L1-L3 depth checks with no CBS-specific code — both handlers duck-type the scoped aspect</t>
+          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2102,7 +2102,7 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>B-01e</t>
+          <t>B-01b</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -2112,12 +2112,12 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Masters — list screens</t>
+          <t>Masters — promotion queue (mdg)</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
+          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
+          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2139,7 +2139,7 @@
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>B-01f</t>
+          <t>B-01c</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -2149,12 +2149,12 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Masters — object page</t>
+          <t>Masters — validation rules</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
+          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
+          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2176,7 +2176,7 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>B-01h</t>
+          <t>B-01d</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2186,12 +2186,12 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Masters — draft editing</t>
+          <t>Masters — remaining entities catalogued</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
+          <t>CBS library, productivity and consumption norms, templates, material mirror added to the authorization catalogue</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
@@ -2201,19 +2201,19 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
+          <t>CBS library picked up isolation, promotion and L1-L3 depth checks with no CBS-specific code — both handlers duck-type the scoped aspect</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>B-01g</t>
+          <t>B-01e</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Masters — productivity and consumption norms</t>
+          <t>Masters — list screens</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>One screen, two tabs; plus a material branch in the resource tree so consumption norms attach to materials rather than equipment</t>
+          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>4 productivity norms with crew composition, 3 consumption norms with wastage; group 105 kg/m3 rebar against INFC's own 112 kg for coastal detailing</t>
+          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2250,7 +2250,7 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>B-02a</t>
+          <t>B-01f</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2260,12 +2260,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Templates — model and instantiation</t>
+          <t>Masters — object page</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2287,7 +2287,7 @@
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>B-02b</t>
+          <t>B-01h</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2297,34 +2297,34 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Templates — screen</t>
+          <t>Masters — draft editing</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>List and object page; instantiate action from the UI rather than the API</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-01g</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2334,34 +2334,34 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Masters — productivity and consumption norms</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>One screen, two tabs; plus a material branch in the resource tree so consumption norms attach to materials rather than equipment</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
+          <t>4 productivity norms with crew composition, 3 consumption norms with wastage; group 105 kg/m3 rebar against INFC's own 112 kg for coastal detailing</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-02a</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2371,34 +2371,34 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Templates — model and instantiation</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
+          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-02b</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2408,34 +2408,34 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Templates — screen</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>List plus an instantiate dialog offering the projects the user may see; refusal surfaces the service's own message</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Driven through the UI: TPL-HIGHRISE into PRJ-002 created 7 CBS nodes and 6 planned resources; a second run raised the refusal</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>Object page for a template still to do</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-03a</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2445,12 +2445,12 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>Project master, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -2465,14 +2465,14 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>Next block; S/4 tenant (Q-09) becomes the blocker for the mirror</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2482,12 +2482,12 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -2502,14 +2502,14 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2519,12 +2519,12 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -2539,14 +2539,14 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2556,12 +2556,12 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -2576,14 +2576,14 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2593,12 +2593,12 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -2613,71 +2613,71 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>MTA builds a deployable archive</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>First Cloud Foundry deployment</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
-        </is>
-      </c>
-      <c r="E55" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -2687,29 +2687,29 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
+          <t>Client billing, variations, payment certificates</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -2724,42 +2724,190 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
+          <t>B-09</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Plant Department</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>Last per your sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>MTA builds a deployable archive</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>First Cloud Foundry deployment</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E61" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
+      <c r="F61" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="G61" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -2780,7 +2928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3432,6 +3580,117 @@
       <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>D-17</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>The project is mastered in KONSTRYX, not in S/4</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Your instruction. A project is created in KONSTRYX and synchronised outward to S/4, or brought in from Primavera P6. This reverses the KONSTRYX-as-reader assumption for the project object specifically; procurement and finance stay S/4-owned</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>High — prj.Project is currently @readonly as an S/4 mirror and must become writable with outbound sync and an unsynchronised state visible in the UI</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>D-18</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Every master and transaction gets upload and download</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Your instruction. Excel import/export as a first-class capability rather than per-screen bespoke work, and the route by which projects arrive from P6</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>High — a shared import/export framework touching every module; needs template definition, validation, error reporting and a staging area</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>D-19</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Flexible approval workflow on every object</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Your instruction. Extends the approval framework already modelled from budgets to all masters and transactions, with the workflow configurable rather than coded</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Engine built and verified. Value bands, approver personas, separation of duties, delegation and withdrawal are all configuration. Remaining: the inbox screen and wiring submit into each object's lifecycle</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Decided — engine done</t>
         </is>
       </c>
     </row>
@@ -3674,17 +3933,17 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>The framework is built but has no content. Needs real thresholds per object per company</t>
+          <t>The engine is built and two starting schemes ship with it — Budget (100k / 1m) and Resource Request (250k / 1m), both with no approver persona set because personas are yours to name. Those thresholds are a placeholder I invented; they are not your policy</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Per object type: steps, approver persona, amount bands</t>
+          <t>Confirm or replace the thresholds, and name the persona that approves each step. All of it is configurable in the app — no redeploy</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>F-02 Approval engine</t>
+          <t>F-02 is done and running on these defaults</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -3694,7 +3953,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Before Budgeting</t>
+          <t>Before the first client demo</t>
         </is>
       </c>
     </row>
@@ -3891,22 +4150,22 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud dev tenant access</t>
+          <t>S/4 dev tenant — what is actually needed (merges the old S-15)</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>No connector can be built or validated without it. Named as a prerequisite in the phase plan</t>
+          <t>Nothing S/4-facing can be built or tested without it. Four concrete things: (1) the tenant API host, e.g. https://myNNNNNN-api.s4hana.cloud.sap; (2) a communication user with password, or a client certificate; (3) communication arrangements activated - SAP_COM_0308 first, since the project now syncs OUTWARD; (4) a named S/4 administrator who can set those up and re-activate them when they expire</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Provide tenant + communication arrangements</t>
+          <t>Provide all four, or confirm the connector is deferred</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>Project sync (D-17), all S/4 mirrors</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -3916,7 +4175,7 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Before Project Setup</t>
+          <t>Before the S/4 connector - NOT blocking upload/download or approvals</t>
         </is>
       </c>
     </row>
@@ -4480,7 +4739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5074,25 +5333,321 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>S/4 dev tenant is on the critical path</t>
+          <t>Merged into Q-09</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>No connector can be built or validated without it, and it is named as a prerequisite in the phase plan</t>
+          <t>Was a duplicate of the S/4 tenant question; the concrete list of what is needed now lives on Q-09</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Secure access before Project Setup</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
+          <t>See Q-09</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>S-16</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>The reader principle now has an exception</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>D-17 makes the project KONSTRYX-mastered while procurement and finance stay S/4-owned. The principle is no longer 'S/4 owns transactions'; it is object by object</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Restate the rule in the product documentation so the exception is deliberate rather than remembered</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>S-17</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>An unsynchronised project is dangerous</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>A project created in KONSTRYX that failed to reach S/4 will still accept requests and budgets that can never post</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Show the unsynchronised state prominently in the UI and block budget release until the S/4 project exists</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>S-18</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Build upload/download once, not per screen</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>D-18 applies to every master and transaction. Bespoke import per screen is how 40 modules end up with 40 different error behaviours</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>One framework: template definition, staging, validation against the same service rules, and an error report the user can correct and re-upload</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>S-19</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Approvals</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>The delivered value bands are mine, not yours</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>The engine ships with Budget at 100k/1m and Resource Request at 250k/1m so it works out of the box. Nobody at Inflexion or a client has agreed those figures, and a demo will show them as if they were policy</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Replace them before any client sees the product. See Q-03</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>S-20</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Approvals</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Separation of duties is on by default</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Someone who cleared step 1 cannot clear step 2 of the same document. In a small contractor one director genuinely is both signatures, so allowChaining exists per step to permit it</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Confirm the default is right for EC&amp;O clients; it is a per-step switch either way</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>S-21</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Approvals</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Nothing yet withdraws an approval when the document changes</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>A resource request approved at AED 2m stays approved if someone later edits it down to 200k, or up. The approval records the amount it was judged on but nothing re-checks it</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Decide per object type whether an edit invalidates an in-flight or completed approval; wire it with F-05</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>S-22</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Approvals</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Editing a scheme mid-flight</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Instances freeze the step number and name at submission, so an in-flight approval survives a scheme edit. It still points at the step definition for the approver persona, and CAP draft activation can renumber those rows</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Confirm the intended behaviour: should a scheme edit affect approvals already running? Today it partly does</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>S-23</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Frameworks</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Content packs now carry references</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Delivered content could previously only hold flat rows, which is why the approval schemes could not ship as content. Packs now resolve a row by natural key at deploy time and match on composite keys</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Use the same mechanism for the EC&amp;O starter pack (S-13) and for delivered personas</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
@@ -5839,7 +6394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6975,6 +7530,117 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>I-29</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Approvals</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>An approval could be raised against an object that does not exist</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>The target is polymorphic - an entity name and a key, not a typed association - so no foreign key would ever object. The approval would sit in an inbox indefinitely pointing at nothing</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Submission now checks the entity is in the model and the row is really there</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>I-30</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>A failing content pack left rows behind that nothing recorded as applied</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Rows were inserted one at a time and the pack's own record written last. When that record failed - a description longer than its column - the rows stayed and the pack looked unapplied</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Each pack now applies in its own change set and is abandoned whole on failure</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>I-31</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Approvals</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>withdraw and delegate returned 501 Not Implemented</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Both actions were declared in CDS without a return type while their handlers set one, which CAP rejects at the protocol layer rather than at build time. Only reachable by calling them - the build was clean</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Declared returns String on both</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
Tracker: attachments done, three new flags
S-25 is the one that matters before a client tenant exists: any authenticated
user can upload any file of any size to any object, with no scanning and no
size cap.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1473,7 +1473,7 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>F-03</t>
+          <t>F-07</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Attachments model</t>
+          <t>Attachments on every object</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Polymorphic on entityName+objectID, media-type content, categories</t>
+          <t>One polymorphic attachment table for all modules; automatic versioning with a supersedes chain; client-configurable categories; a mandatory category blocks approval submission</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1498,19 +1498,19 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>14 checks: v1 then v2 superseding it, PDF streamed in and read back byte-identical, 404 for a missing target, and submission refused until the mandatory drawing was attached</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Upload handler + object store not built</t>
+          <t>fileSize (F-08) and the UI upload control</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>F-04</t>
+          <t>F-08</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1520,12 +1520,12 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Attachment upload + storage</t>
+          <t>Attachment file size</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Object store binding for Cloud Foundry vs HANA LOB</t>
+          <t>fileSize is null — measuring the media stream consumes it, so it needs a counting wrapper on the upload path</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -1540,14 +1540,14 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Decision needed (see Open Decisions)</t>
+          <t>Low priority; display only</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>F-05</t>
+          <t>F-09</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1557,34 +1557,34 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Table personalization store</t>
+          <t>Attachment storage</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>UserVariant entity holding UI5 p13n state per user</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Content sits in the database as LargeBinary. Fine for drawings and permits; a project's photo library is a different question</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Not wired to any table yet</t>
+          <t>Decide before go-live — see S-24</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>F-06</t>
+          <t>F-03</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1594,86 +1594,86 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Table personalization UI wiring</t>
+          <t>Attachments model</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>p13n + VariantManagement on every list screen</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Polymorphic on entityName+objectID, media-type content, categories</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Apply as each screen is built</t>
+          <t>Upload handler + object store not built</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>M-01</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Workflow spine RR-&gt;ADV-&gt;AVC-&gt;RES</t>
+          <t>Attachment upload + storage</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Vertical-agnostic, multi-line, seeded with canonical EQR thread</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Object store binding for Cloud Foundry vs HANA LOB</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Queryable over OData; 5 lines, AED 685,080</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Decision needed (see Open Decisions)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>M-02</t>
+          <t>F-05</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>WBS on request line</t>
+          <t>Table personalization store</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Spec section 6 requires one WBS per line; was missing</t>
+          <t>UserVariant entity holding UI5 p13n state per user</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1683,56 +1683,56 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>3 distinct WBS across the 5 EQR lines</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Not wired to any table yet</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>M-03</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>EQR vertical extension</t>
+          <t>Table personalization UI wiring</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Instances, mob/demob window, own-vs-rental, vendor, operators</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>p13n + VariantManagement on every list screen</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>$expand=equipment,wbs returns all 5 lines resolved</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Apply as each screen is built</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>M-04</t>
+          <t>M-01</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -1742,49 +1742,49 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Chain steps CMT/MOB/OPL/VAR/DMB/CLS</t>
+          <t>Workflow spine RR-&gt;ADV-&gt;AVC-&gt;RES</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Steps 5-10 have no CDS entities at all</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Vertical-agnostic, multi-line, seeded with canonical EQR thread</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
+          <t>Queryable over OData; 5 lines, AED 685,080</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>Part of Project Execution block</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>U-01</t>
+          <t>M-02</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>RR worklist on live OData</t>
+          <t>WBS on request line</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>RequestOverview projection, server-side filters</t>
+          <t>Spec section 6 requires one WBS per line; was missing</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Verified in browser: 4 requests, EQR shows 5 lines / 685,080; EQR filter issues new $batch</t>
+          <t>3 distinct WBS across the 5 EQR lines</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1806,64 +1806,64 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>U-02</t>
+          <t>M-03</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Request detail page on OData</t>
+          <t>EQR vertical extension</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Still reads webapp/model/data.json</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Instances, mob/demob window, own-vs-rental, vendor, operators</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
+          <t>$expand=equipment,wbs returns all 5 lines resolved</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
-        <is>
-          <t>Now unblocked by M-03</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>U-03</t>
+          <t>M-04</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Chain step pages on OData</t>
+          <t>Chain steps CMT/MOB/OPL/VAR/DMB/CLS</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Still read data.json</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Steps 5-10 have no CDS entities at all</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -1873,14 +1873,14 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Blocked by M-04</t>
+          <t>Part of Project Execution block</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>U-04</t>
+          <t>U-01</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -1890,12 +1890,12 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Launchpad intents declared</t>
+          <t>RR worklist on live OData</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
+          <t>RequestOverview projection, server-side filters</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>manifest parses; two inbounds registered</t>
+          <t>Verified in browser: 4 requests, EQR shows 5 lines / 685,080; EQR filter issues new $batch</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -1917,7 +1917,7 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>U-05</t>
+          <t>U-02</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -1927,34 +1927,34 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Launchpad-hosted shell (blend with S/4)</t>
+          <t>Request detail page on OData</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
-        </is>
-      </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Still reads webapp/model/data.json</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Now unblocked by M-03</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>U-06</t>
+          <t>U-03</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -1964,34 +1964,34 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Spaces and Pages navigation</t>
+          <t>Chain step pages on OData</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
+          <t>Still read data.json</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
+          <t>Blocked by M-04</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>U-08</t>
+          <t>U-04</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2001,34 +2001,34 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Split into task-focused apps per document type</t>
+          <t>Launchpad intents declared</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
+          <t>manifest parses; two inbounds registered</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>Register more intents as screens are built</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>U-07</t>
+          <t>U-05</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -2038,12 +2038,12 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Morning Horizon theme</t>
+          <t>Launchpad-hosted shell (blend with S/4)</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
+          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -2053,108 +2053,108 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
+          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>B-01a</t>
+          <t>U-06</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Masters — hybrid scope enforcement</t>
+          <t>Spaces and Pages navigation</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
+          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>B-01b</t>
+          <t>U-08</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Masters — promotion queue (mdg)</t>
+          <t>Split into task-focused apps per document type</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Register more intents as screens are built</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>B-01c</t>
+          <t>U-07</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Masters — validation rules</t>
+          <t>Morning Horizon theme</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
+          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -2164,19 +2164,19 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
+          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>B-01d</t>
+          <t>B-01a</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -2186,12 +2186,12 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Masters — remaining entities catalogued</t>
+          <t>Masters — hybrid scope enforcement</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>CBS library, productivity and consumption norms, templates, material mirror added to the authorization catalogue</t>
+          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>CBS library picked up isolation, promotion and L1-L3 depth checks with no CBS-specific code — both handlers duck-type the scoped aspect</t>
+          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2213,7 +2213,7 @@
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>B-01e</t>
+          <t>B-01b</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Masters — list screens</t>
+          <t>Masters — promotion queue (mdg)</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
+          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
+          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -2250,7 +2250,7 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>B-01f</t>
+          <t>B-01c</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2260,12 +2260,12 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Masters — object page</t>
+          <t>Masters — validation rules</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
+          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
+          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2287,7 +2287,7 @@
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>B-01h</t>
+          <t>B-01d</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2297,12 +2297,12 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Masters — draft editing</t>
+          <t>Masters — remaining entities catalogued</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
+          <t>CBS library, productivity and consumption norms, templates, material mirror added to the authorization catalogue</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -2312,19 +2312,19 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
+          <t>CBS library picked up isolation, promotion and L1-L3 depth checks with no CBS-specific code — both handlers duck-type the scoped aspect</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>B-01g</t>
+          <t>B-01e</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2334,12 +2334,12 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Masters — productivity and consumption norms</t>
+          <t>Masters — list screens</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>One screen, two tabs; plus a material branch in the resource tree so consumption norms attach to materials rather than equipment</t>
+          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>4 productivity norms with crew composition, 3 consumption norms with wastage; group 105 kg/m3 rebar against INFC's own 112 kg for coastal detailing</t>
+          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2361,7 +2361,7 @@
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>B-02a</t>
+          <t>B-01f</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2371,12 +2371,12 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Templates — model and instantiation</t>
+          <t>Masters — object page</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2398,7 +2398,7 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>B-02b</t>
+          <t>B-01h</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2408,12 +2408,12 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Templates — screen</t>
+          <t>Masters — draft editing</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>List plus an instantiate dialog offering the projects the user may see; refusal surfaces the service's own message</t>
+          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -2423,19 +2423,19 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>Driven through the UI: TPL-HIGHRISE into PRJ-002 created 7 CBS nodes and 6 planned resources; a second run raised the refusal</t>
+          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Object page for a template still to do</t>
+          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>B-03a</t>
+          <t>B-01g</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -2445,34 +2445,34 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Masters — productivity and consumption norms</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Project master, WBS, CBS instance; S/4 Enterprise Project mirror</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>One screen, two tabs; plus a material branch in the resource tree so consumption norms attach to materials rather than equipment</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
+          <t>4 productivity norms with crew composition, 3 consumption norms with wastage; group 105 kg/m3 rebar against INFC's own 112 kg for coastal detailing</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
-        <is>
-          <t>Next block; S/4 tenant (Q-09) becomes the blocker for the mirror</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-02a</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -2482,34 +2482,34 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Templates — model and instantiation</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
+          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-02b</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -2519,34 +2519,34 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Templates — screen</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>List plus an instantiate dialog offering the projects the user may see; refusal surfaces the service's own message</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Driven through the UI: TPL-HIGHRISE into PRJ-002 created 7 CBS nodes and 6 planned resources; a second run raised the refusal</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>Object page for a template still to do</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-03a</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -2556,12 +2556,12 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>Project master, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -2576,14 +2576,14 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>Next block; S/4 tenant (Q-09) becomes the blocker for the mirror</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2593,12 +2593,12 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -2613,14 +2613,14 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
@@ -2630,12 +2630,12 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
@@ -2650,14 +2650,14 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -2667,12 +2667,12 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -2687,14 +2687,14 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
@@ -2704,12 +2704,12 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -2724,14 +2724,14 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -2741,12 +2741,12 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
@@ -2761,71 +2761,71 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>MTA builds a deployable archive</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
-        </is>
-      </c>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>First Cloud Foundry deployment</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
-        </is>
-      </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Client billing, variations, payment certificates</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
@@ -2835,29 +2835,29 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>Plant Department</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
+          <t>Equipment, fleet, scaffolding/formwork</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -2872,42 +2872,153 @@
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Needs S/4 dev tenant access</t>
+          <t>Last per your sequence</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>MTA builds a deployable archive</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>First Cloud Foundry deployment</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Mirror entities exist; no connector, no destination wiring</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>Needs S/4 dev tenant access</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C61" s="7" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D64" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr">
+      <c r="E64" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F61" s="7" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="G64" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -4739,7 +4850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5619,35 +5730,146 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
+          <t>S-24</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Attachments</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Attachment content is stored in the database</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>LargeBinary in HANA is right for the documents that carry legal weight — drawings, permits, signed variations — because they are backed up and restored with the data they belong to. It is the wrong home for thousands of site photographs</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Decide whether photo-heavy objects go to an object store instead. It is a per-category switch if decided before volume builds up, and a migration afterwards</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>S-25</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Attachments</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Nothing scans uploads or limits their size</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Any authenticated user can upload any file of any size to any object. On a client tenant that is both a malware route and a storage risk</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Add a size cap and virus scanning before the first client upload. SAP BTP has a Malware Scanning service; the size cap is configuration</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>S-26</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Attachments</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Deleting an attachment breaks the version chain</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>supersedes points at the previous version. Deleting a middle version leaves the chain dangling, and deleting the document someone approved against destroys the evidence</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Block deletion of a superseded version, or of anything attached to a closed approval; mark as obsolete instead</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>S-23</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Frameworks</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Content packs now carry references</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Delivered content could previously only hold flat rows, which is why the approval schemes could not ship as content. Packs now resolve a row by natural key at deploy time and match on composite keys</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>Use the same mechanism for the EC&amp;O starter pack (S-13) and for delivered personas</t>
         </is>
       </c>
-      <c r="F28" s="11" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Tracker: regenerate — S/4 connector done, reservation overview (U-09) added
The .xlsx had drifted behind the generator script (S/4 connector and
Q-09p closure were already in build_tracker.py but nobody re-ran it).
Regenerated, added U-09 for the reservation overview rebuild, and
corrected D-02's stale Not started to Done (project scenario only).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Status Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Work Items" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Decisions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Open Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Planned Sequence" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Suggestions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Options Considered" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Issues" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work Items" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planned Sequence" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suggestions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options Considered" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1214,96 +1214,96 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>A-04</t>
+          <t>PS-01</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Write-path input-data check</t>
+          <t>Projects and WBS mastered in KONSTRYX</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Reject CREATE/UPDATE carrying a project outside the user's scope</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Draft-enabled and writable; code uniqueness, date agreement, company required, hierarchy cycle guard; sync state protected from hand-editing on both the active record and the draft</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>20 checks: a new project activates NOT_SENT; release refuses a project with no WBS, queues one that has it, refuses a second release; the connector callback moves it FAILED then SENT with the refusal text and attempt count kept</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Validate after Project Setup exists</t>
+          <t>Primavera import (PS-03)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>A-05</t>
+          <t>PS-02</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Administration UI</t>
+          <t>Outbound sync aspect</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>S/4-like screens to maintain personas, grants, assignments</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>s4outbound, separate from s4mirror because the two directions need opposite defaults — a project created here starts NOT_SENT, not OK</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Seeded projects read SENT; a new one reads NOT_SENT</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Part of Masters/Admin UI block</t>
+          <t>The connector itself needs Q-09</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>F-01</t>
+          <t>PS-03</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Approval framework model</t>
+          <t>Primavera P6 project import</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Schemes per object type, ordered steps, approver persona, value bands, runtime instances</t>
+          <t>P6 XML export creates the project and its WBS tree in one file, through ProjectService so the same validation applies. No PARTIAL mode: a tree only means anything whole. DTDs and external entities switched off on the parser</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1313,34 +1313,34 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>15 checks: dry run changes nothing; a child WBS parents correctly despite preceding its parent in the file; re-import leaves exactly one project and four elements; an XXE attempt is refused and leaks nothing</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P6 activities and the schedule itself are not imported — see S-31</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>F-02</t>
+          <t>PL-02</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Approval engine</t>
+          <t>WBS distribution by template</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Instantiate on submit, match value bands, advance steps, enforce approver persona and separation of duties, delegate, withdraw, audit</t>
+          <t>TPL-SINGLE / TPL-FLOORS / TPL-ZONES: one decision covers many lines; weighted split with the rounding residue on the last target so VAL-02 passes to the third decimal; re-running replaces rather than stacks; template and splitBasis on every allocation row</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -1350,108 +1350,108 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>28 checks against the running service: bands select 1/2/3 steps at 50k/300k/2m; out-of-order, double, reasonless and same-person decisions all refused; persona configured through the admin API then enforced</t>
+          <t>18 checks: 40/35/25 gives 480/420/300 exactly; thirds of 1000 keep the millimetre; the bulk path takes the whole bill in one decision and the gate flips to Pass</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Inbox screen (F-04) and per-object wiring (F-05)</t>
+          <t>Distribute dialog on the workbench UI</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>F-04</t>
+          <t>PL-03</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Approval inbox screen</t>
+          <t>Cost Mapping workbench</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>The steps awaiting the signed-in user, with approve, reject and delegate</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Four step tiles (CBS / WBS / Resources / Gate) and an exceptions-only queue with reasons and modest CBS suggestions; Generate Budget Lines disabled while the gate fails, tooltip names why (UI-04). The queue names unrated resources as work items instead of a generate treadmill</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Browser-verified: 9 honest exceptions across three reasons on the canonical fixture; console clean</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>With the UI rebuild</t>
+          <t>Distribute + rate-fix flows from the queue rows</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>F-05</t>
+          <t>UI-01</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Wire submit into each object's lifecycle</t>
+          <t>Projects, BOQ and assigned-CBS screens</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Today the caller chooses when to submit. Each document type should move to 'In Approval' on submit and act on the outcome</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Projects worklist (workplace group, not Masters); BOQ with the canonical F.1 lines, contract vs budget qty side by side, build-up drill, Generate Build-up and Check Gate actions; assigned-CBS screen showing the node, its recipe norms with company variants, and its bill lines</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Browser-verified: pile-cap shows all 7 published lines summing 1,198.95/m3; the 03.20 link popover leads with the assigned node; console clean</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Per module as each is built</t>
+          <t>Cost Mapping workbench (exceptions only, UI-01 of the spec) is next</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>F-06</t>
+          <t>UI-02</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Content pack references</t>
+          <t>S/4-style object links, per-user configurable</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Packs can name another row instead of its UUID, and match on composite natural keys; each pack applies atomically</t>
+          <t>An object key is a hyperlink; one target navigates, several open a popover; which targets appear is each user's own choice, persisted through UserVariants. Transaction targets lead; masters are secondary</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1461,34 +1461,34 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>APPROVAL_SCHEMES resolves auth objects and its own schemes at deploy time: 6 rows inserted</t>
+          <t>PRJ-001 offers BOQ + Resource Requests; 03.20 offers Assigned CBS + Library</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Roll the registry across every remaining screen with task #12</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>F-07</t>
+          <t>D-23x</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Attachments on every object</t>
+          <t>Canonical mockup data seeded (spec F.1)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>One polymorphic attachment table for all modules; automatic versioning with a supersedes chain; client-configurable categories; a mandatory category blocks approval submission</t>
+          <t>03.10/03.20/03.30 leaves with grade on the attached material row; MP-CIV-CAR-SK-G1 with ALL 1.13 / INFC 1.25 / PMI 0.95; the pile-cap 7-line build-up as IMPORTED at the published figures</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1498,19 +1498,19 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>14 checks: v1 then v2 superseding it, PDF streamed in and read back byte-identical, 404 for a missing target, and submission refused until the mandatory drawing was attached</t>
+          <t>Per-m3 sum 1,198.95 matches the wireframe to the fils; OPEN-05 residual seeded as published, not invented into agreement</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>fileSize (F-08) and the UI upload control</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>F-08</t>
+          <t>F-11</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1520,49 +1520,49 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Attachment file size</t>
+          <t>A person can read their own import history</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>fileSize is null — measuring the media stream consumes it, so it needs a counting wrapper on the upload path</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>MyImportRuns and MyImportRows, narrowed to what that person uploaded</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
+          <t>The importing user reads back three runs including 'line 1: Project code DHV-P3 already exists'</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>Low priority; display only</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>F-09</t>
+          <t>A-04</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Attachment storage</t>
+          <t>Write-path input-data check</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Content sits in the database as LargeBinary. Fine for drawings and permits; a project's photo library is a different question</t>
+          <t>Reject CREATE/UPDATE carrying a project outside the user's scope</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -1577,51 +1577,51 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Decide before go-live — see S-24</t>
+          <t>Validate after Project Setup exists</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>F-03</t>
+          <t>A-05</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Attachments model</t>
+          <t>Administration UI</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Polymorphic on entityName+objectID, media-type content, categories</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>S/4-like screens to maintain personas, grants, assignments</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Upload handler + object store not built</t>
+          <t>Part of Masters/Admin UI block</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>F-04</t>
+          <t>F-01</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1631,34 +1631,34 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Attachment upload + storage</t>
+          <t>Approval framework model</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Object store binding for Cloud Foundry vs HANA LOB</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Schemes per object type, ordered steps, approver persona, value bands, runtime instances</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
+          <t>Compiles; exposed on /collaboration</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>Decision needed (see Open Decisions)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>F-05</t>
+          <t>F-02</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1668,12 +1668,12 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Table personalization store</t>
+          <t>Approval engine</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>UserVariant entity holding UI5 p13n state per user</t>
+          <t>Instantiate on submit, match value bands, advance steps, enforce approver persona and separation of duties, delegate, withdraw, audit</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1683,19 +1683,19 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Compiles; exposed on /collaboration</t>
+          <t>28 checks against the running service: bands select 1/2/3 steps at 50k/300k/2m; out-of-order, double, reasonless and same-person decisions all refused; persona configured through the admin API then enforced</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Not wired to any table yet</t>
+          <t>Inbox screen (F-04) and per-object wiring (F-05)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>F-06</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1705,12 +1705,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Table personalization UI wiring</t>
+          <t>Approval inbox screen</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>p13n + VariantManagement on every list screen</t>
+          <t>The steps awaiting the signed-in user, with approve, reject and delegate</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -1725,66 +1725,66 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Apply as each screen is built</t>
+          <t>With the UI rebuild</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>M-01</t>
+          <t>F-05</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Workflow spine RR-&gt;ADV-&gt;AVC-&gt;RES</t>
+          <t>Wire submit into each object's lifecycle</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Vertical-agnostic, multi-line, seeded with canonical EQR thread</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Today the caller chooses when to submit. Each document type should move to 'In Approval' on submit and act on the outcome</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Queryable over OData; 5 lines, AED 685,080</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Per module as each is built</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>M-02</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>WBS on request line</t>
+          <t>Content pack references</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Spec section 6 requires one WBS per line; was missing</t>
+          <t>Packs can name another row instead of its UUID, and match on composite natural keys; each pack applies atomically</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>3 distinct WBS across the 5 EQR lines</t>
+          <t>APPROVAL_SCHEMES resolves auth objects and its own schemes at deploy time: 6 rows inserted</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -1806,22 +1806,22 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>M-03</t>
+          <t>F-07</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>EQR vertical extension</t>
+          <t>Attachments on every object</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Instances, mob/demob window, own-vs-rental, vendor, operators</t>
+          <t>One polymorphic attachment table for all modules; automatic versioning with a supersedes chain; client-configurable categories; a mandatory category blocks approval submission</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -1831,34 +1831,34 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>$expand=equipment,wbs returns all 5 lines resolved</t>
+          <t>14 checks: v1 then v2 superseding it, PDF streamed in and read back byte-identical, 404 for a missing target, and submission refused until the mandatory drawing was attached</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>fileSize (F-08) and the UI upload control</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>M-04</t>
+          <t>F-08</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Data model</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Chain steps CMT/MOB/OPL/VAR/DMB/CLS</t>
+          <t>Attachment file size</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Steps 5-10 have no CDS entities at all</t>
+          <t>fileSize is null — measuring the media stream consumes it, so it needs a counting wrapper on the upload path</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -1873,29 +1873,29 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Part of Project Execution block</t>
+          <t>Low priority; display only</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>U-01</t>
+          <t>M-10</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Masters</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>RR worklist on live OData</t>
+          <t>Rate master complete</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>RequestOverview projection, server-side filters</t>
+          <t>Draft-maintainable rates and norms; rateOn(resource, date, company) resolves which rate is in force — latest start on or before the date, company beating group; norms validated (no zero output, no 140% wastage, effective-date clashes on the full recipe key)</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Verified in browser: 4 requests, EQR shows 5 lines / 685,080; EQR filter issues new $batch</t>
+          <t>17 checks</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -1917,96 +1917,96 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>U-02</t>
+          <t>PS-04</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Request detail page on OData</t>
+          <t>BOQ import and arithmetic</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Still reads webapp/model/data.json</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>amount always qty x rate, never accepted from the caller; header equals sum of lines; all-or-nothing import that also catches duplicates within the file; re-import replaces</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
+          <t>20 checks incl. a bad bill refused whole</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>Now unblocked by M-03</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>U-03</t>
+          <t>PS-05</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Chain step pages on OData</t>
+          <t>Project CBS and allocation</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Still read data.json</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>instantiateCBS copies the library (refuses a second run); allocate joins bill to WBS+CBS with an over-allocation guard and cross-project refusal; CBS nodes carry allocated value at bill rate</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
+          <t>700+500 of a 1200 line to exactly 100%; the repeated 700 refused</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>Blocked by M-04</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>U-04</t>
+          <t>PL-01</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Launchpad intents declared</t>
+          <t>Resource build-up from CBS recipes</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
+          <t>Norms carry the wireframe key (Resource x Linked CBS x Activity x Company); a BOQ line resolves through its CBS leaf; difficulty on top of productivity only, never the master norm (KX-BUD-014); MANUAL rows survive regeneration and are counted as defects; coverage report: recipe-found / manual / no-recipe / unmapped / rate-missing</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -2016,34 +2016,34 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>manifest parses; two inbounds registered</t>
+          <t>16 checks: 1230 m3 (2.5% wastage), 110 hr (std 12/hr x 110%), INFC override wins</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Activity Code Library difficulty resolution deferred — difficulty is a call parameter today</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>U-05</t>
+          <t>EX-01</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Execution</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Launchpad-hosted shell (blend with S/4)</t>
+          <t>RR to RES chain engine</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
+          <t>submit prices lines from the rate master and refuses unpriced resources; approval outcome moves the document (F-05, generic); advisory line-by-line with rationale; AVC documents KONSTRYX-side commitments honestly, S/4 ATP slots in later; reservation encumbers the approved value; StatusHistory + DocumentLinks throughout</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -2053,145 +2053,145 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
+          <t>28 checks; every shortcut refused with the missing step named</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>S/4 ATP behind the same document (Q-09)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>U-06</t>
+          <t>B-06x</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Spaces and Pages navigation</t>
+          <t>Budget engine</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>At risk</t>
+          <t>Generated from the priced build-up by CBS x cost nature (six); refuses unpriced resources whole; approval via BUD-STD; baseline makes the ledger the only door (PATCH on a baselined amount answers 403); zero-sum paired SHIFT with mandatory reason; refreshControl pulls open reservation encumbrance into the control record</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
+          <t>25 checks; line amount == sum of its ledger entries asserted per line</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
+          <t>Risk Transfer and Variation documents feeding their ledger categories</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>U-08</t>
+          <t>F-10</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Split into task-focused apps per document type</t>
+          <t>Per-user table personalization</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Saved column sets, filters, sorts and groupings per user per table; one default each; administrator-published variants readable by all</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>18 checks: two users hold the same variant name on the same table and see only their own; a new default clears the previous one and leaves other users alone; writing to someone else's answers 404, not 403, so the key is not confirmed</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Register more intents as screens are built</t>
+          <t>UI wiring comes with the screen rebuild</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>U-07</t>
+          <t>F-09</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Morning Horizon theme</t>
+          <t>Attachment storage</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Content sits in the database as LargeBinary. Fine for drawings and permits; a project's photo library is a different question</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
+          <t>Decide before go-live — see S-24</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>B-01a</t>
+          <t>F-03</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Masters — hybrid scope enforcement</t>
+          <t>Attachments model</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
+          <t>Polymorphic on entityName+objectID, media-type content, categories</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
@@ -2201,71 +2201,71 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Upload handler + object store not built</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>B-01b</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Masters — promotion queue (mdg)</t>
+          <t>Attachment upload + storage</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Object store binding for Cloud Foundry vs HANA LOB</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Decision needed (see Open Decisions)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>B-01c</t>
+          <t>F-05</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Masters — validation rules</t>
+          <t>Table personalization store</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
+          <t>UserVariant entity holding UI5 p13n state per user</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -2275,71 +2275,71 @@
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
+          <t>Compiles; exposed on /collaboration</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Not wired to any table yet</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>B-01d</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Masters — remaining entities catalogued</t>
+          <t>Table personalization UI wiring</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>CBS library, productivity and consumption norms, templates, material mirror added to the authorization catalogue</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>p13n + VariantManagement on every list screen</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>CBS library picked up isolation, promotion and L1-L3 depth checks with no CBS-specific code — both handlers duck-type the scoped aspect</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Apply as each screen is built</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>B-01e</t>
+          <t>M-01</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Masters — list screens</t>
+          <t>Workflow spine RR-&gt;ADV-&gt;AVC-&gt;RES</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
+          <t>Vertical-agnostic, multi-line, seeded with canonical EQR thread</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
+          <t>Queryable over OData; 5 lines, AED 685,080</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2361,22 +2361,22 @@
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>B-01f</t>
+          <t>M-02</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Masters — object page</t>
+          <t>WBS on request line</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
+          <t>Spec section 6 requires one WBS per line; was missing</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
+          <t>3 distinct WBS across the 5 EQR lines</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2398,22 +2398,22 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>B-01h</t>
+          <t>M-03</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Masters — draft editing</t>
+          <t>EQR vertical extension</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
+          <t>Instances, mob/demob window, own-vs-rental, vendor, operators</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -2423,71 +2423,71 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
+          <t>$expand=equipment,wbs returns all 5 lines resolved</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>B-01g</t>
+          <t>M-04</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Data model</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Masters — productivity and consumption norms</t>
+          <t>Chain steps CMT/MOB/OPL/VAR/DMB/CLS</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>One screen, two tabs; plus a material branch in the resource tree so consumption norms attach to materials rather than equipment</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Steps 5-10 have no CDS entities at all</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>4 productivity norms with crew composition, 3 consumption norms with wastage; group 105 kg/m3 rebar against INFC's own 112 kg for coastal detailing</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Part of Project Execution block</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>B-02a</t>
+          <t>U-01</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Templates — model and instantiation</t>
+          <t>RR worklist on live OData</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+          <t>RequestOverview projection, server-side filters</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+          <t>Verified in browser: 4 requests, EQR shows 5 lines / 685,080; EQR filter issues new $batch</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2509,64 +2509,64 @@
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>B-02b</t>
+          <t>U-02</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Templates — screen</t>
+          <t>Request detail page on OData</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>List plus an instantiate dialog offering the projects the user may see; refusal surfaces the service's own message</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Still reads webapp/model/data.json</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Driven through the UI: TPL-HIGHRISE into PRJ-002 created 7 CBS nodes and 6 planned resources; a second run raised the refusal</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>Object page for a template still to do</t>
+          <t>Now unblocked by M-03</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>B-03a</t>
+          <t>U-03</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Chain step pages on OData</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Project master, WBS, CBS instance; S/4 Enterprise Project mirror</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Still read data.json</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
@@ -2576,140 +2576,140 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Next block; S/4 tenant (Q-09) becomes the blocker for the mirror</t>
+          <t>Blocked by M-04</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>U-04</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Launchpad intents declared</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>crossNavigation inbounds for KonstryxResourceRequest and KonstryxReservation</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
+          <t>manifest parses; two inbounds registered</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
-        <is>
-          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>U-05</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Launchpad-hosted shell (blend with S/4)</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>App shell removed: root view is now the NavContainer alone. Launchpad supplies header, search, user menu, theme</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
+          <t>Verified in browser as daud: worklist renders with no app chrome, 4 of 5 requests correctly scoped, EQR at AED 685,080</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>U-06</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Spaces and Pages navigation</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>flp.html + flpSite.json written: CDM 3.1 site, one space, one page, two intent tiles</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>At risk</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Site JSON authored against the runtime's own sandboxSite.json schema</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>Sandbox bootstrap fails reading a null script element; finish or verify on real BTP instead</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>U-08</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Split into task-focused apps per document type</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>S/4 pattern is one app per task, reached from a tile. Currently one app with in-app routing across ten document types</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -2724,88 +2724,88 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>Register more intents as screens are built</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>U-09</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Reservation overview — chain progress + honest S/4 status</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>You flagged the old screen as poorly designed with no visible chain progress or S/4 truth. Rebuilt: reservationOverview action computes steps-done/steps-pending across the full ten-step chain from live documents (RR, advisory, AVC, RES, closure); the header states per integration path what is actually connected — project sync LIVE, CMT/procurement/BP mirror not wired — and every row carries its own project's sync state</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Verified in browser: RES-2026-0188 reads 4 of 10 steps, pending CMT/MOB/OPL/VAR/DMB/CLS listed explicitly; full regression 13 suites / 261 checks green</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>CMT connector, once S/4 PS commitment posting is in scope</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>U-07</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Morning Horizon theme</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-01a</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -2815,34 +2815,34 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Masters — hybrid scope enforcement</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
+          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="inlineStr">
-        <is>
-          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-01b</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -2852,49 +2852,49 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Masters — promotion queue (mdg)</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
+          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G60" s="7" t="inlineStr">
-        <is>
-          <t>Last per your sequence</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-01c</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>MTA builds a deployable archive</t>
+          <t>Masters — validation rules</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
@@ -2916,109 +2916,738 @@
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>B-01d</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>First Cloud Foundry deployment</t>
+          <t>Masters — remaining entities catalogued</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
-        </is>
-      </c>
-      <c r="E62" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>CBS library, productivity and consumption norms, templates, material mirror added to the authorization catalogue</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
+          <t>CBS library picked up isolation, promotion and L1-L3 depth checks with no CBS-specific code — both handlers duck-type the scoped aspect</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G62" s="7" t="inlineStr">
-        <is>
-          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>B-01e</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>Masters — list screens</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Mirror entities exist; no connector, no destination wiring</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
+          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G63" s="7" t="inlineStr">
-        <is>
-          <t>Needs S/4 dev tenant access</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
+          <t>B-01f</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Masters — object page</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>B-01h</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Masters — draft editing</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>B-01g</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Masters — productivity and consumption norms</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>One screen, two tabs; plus a material branch in the resource tree so consumption norms attach to materials rather than equipment</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>4 productivity norms with crew composition, 3 consumption norms with wastage; group 105 kg/m3 rebar against INFC's own 112 kg for coastal detailing</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>B-02a</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Templates — model and instantiation</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>B-02b</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Templates — screen</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>List plus an instantiate dialog offering the projects the user may see; refusal surfaces the service's own message</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>Driven through the UI: TPL-HIGHRISE into PRJ-002 created 7 CBS nodes and 6 planned resources; a second run raised the refusal</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>Object page for a template still to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>B-03a</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Project Setup</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Project master, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>Next block; S/4 tenant (Q-09) becomes the blocker for the mirror</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>B-02</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Templates</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Project templates: CBS tree + default resources</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>After Masters</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>B-03</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Project Setup</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>After Templates</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>B-04</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Uploads</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Highest-risk item in the sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>B-05</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Project Planning</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Activity layer, native entity + P6 adapter</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>After Uploads</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>B-06</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Budgeting</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>After Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>B-07</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Project Execution</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>After Budgeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>B-08</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Project Commercial</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Client billing, variations, payment certificates</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>After Execution</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>B-09</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Plant Department</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>Last per your sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>MTA builds a deployable archive</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>First Cloud Foundry deployment</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>S4Connection (credentials, CSRF handshake) + S4ProjectConnector (project + WBS push to API_ENTERPRISE_PROJECT_SRV) built and run live against my401381: KX-S4-001 created via release -&gt; sync, confirmed by independent read-back (profile YP05)</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>D-17 loop ran live on the tenant; see Q-09p</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>Scoped to the project scenario only — procurement, finance and BP mirror connectors are not built; BTP destination replaces S4Connection at deployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="B81" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
+      <c r="C81" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D64" s="7" t="inlineStr">
+      <c r="D81" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr">
+      <c r="E81" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
+      <c r="F81" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G81" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -3039,7 +3668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3771,35 +4400,146 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
+          <t>D-22</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>SPEC-planning-budget.md adopted as the planning/budget contract</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Your handover of the full spec. Deltas implemented: derived netRate with inbound ignored (CALC-01), crew expansion with hours multiplied not divided (CALC-02/UT-09), rate-missing writes no build-up line (IT-08), budgetQty vs contractQty never crossed (CALC-05), difficultySrc recorded, resourceAffinity removed (RG-02), and the KX-GOV-002 gate with VAL-01..07 wired into budget generation as 409 GATE_FAILED</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Deliberately deferred, per the spec's own open items: CALC-03 activity tiers (no Activity entity yet), the four-class roll-up (OPEN-01/02 unpinned), budgetQty derivation (OPEN-04), crew role-to-resource mapping (undefined in the spec)</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>D-20</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Cost nature is six, the ledger is four, and they never meet</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Your wireframe answer: cost nature = the six verticals (MR, MPR, EQR, VR, SF, SC), computed from the resource build-up; the Budget Ledger four (Original / Shift / Risk Transfer / Variation, KX-BUD-004) is a movement taxonomy computed from ledger entries. My earlier four-category cost framing was wrong and is retired</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Both implemented: budget lines carry the six; every movement is one ledger entry in one of the four</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>D-21</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Build-up recipes are keyed on the CBS leaf</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Your wireframe answer: Resource x Linked CBS x Activity x Company. A BOQ line resolves through its CBS leaf; nobody keys resources per line; MANUAL build-up is a flagged exception awaiting a recipe, not a way of working</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Implemented, incl. the governance consequence: two lines on one leaf share one recipe, so spec variance needs a distinct leaf or activity code</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
           <t>D-19</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Flexible approval workflow on every object</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Your instruction. Extends the approval framework already modelled from budgets to all masters and transactions, with the workflow configurable rather than coded</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>You</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Engine built and verified. Value bands, approver personas, separation of duties, delegation and withdrawal are all configuration. Remaining: the inbox screen and wiring submit into each object's lifecycle</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>Decided — engine done</t>
         </is>
@@ -3820,7 +4560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4256,64 +4996,64 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Q-09</t>
+          <t>Q-09p</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>S/4 dev tenant — what is actually needed (merges the old S-15)</t>
+          <t>S/4 tenant my401381 - RESOLVED for projects</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Nothing S/4-facing can be built or tested without it. Four concrete things: (1) the tenant API host, e.g. https://myNNNNNN-api.s4hana.cloud.sap; (2) a communication user with password, or a client certificate; (3) communication arrangements activated - SAP_COM_0308 first, since the project now syncs OUTWARD; (4) a named S/4 administrator who can set those up and re-activate them when they expire</t>
+          <t>Communication user + arrangements SAP_COM_0308/0008 active. The connector ran live: KX-S4-001 created in the tenant from KONSTRYX through release -&gt; sync, confirmed by an independent read (profile YP05). Remaining: WBS element read-back navigation name; the other scenarios (procurement, finance) as their modules need them</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Provide all four, or confirm the connector is deferred</t>
+          <t>Rotate the credential that transited chat transcripts when convenient; move to a BTP destination at deployment</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Project sync (D-17), all S/4 mirrors</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>S/4 connector - project scenario DONE</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Before the S/4 connector - NOT blocking upload/download or approvals</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Q-10</t>
+          <t>Q-09</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Scope re-baseline: personalization + attachments + approvals on every screen</t>
+          <t>S/4 dev tenant — what is actually needed (merges the old S-15)</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Wireframe v12 is 41 modules / 434 screens. The 22-week MVP plan with 1 UI5 developer does not carry this</t>
+          <t>Nothing S/4-facing can be built or tested without it. Four concrete things: (1) the tenant API host, e.g. https://myNNNNNN-api.s4hana.cloud.sap; (2) a communication user with password, or a client certificate; (3) communication arrangements activated - SAP_COM_0308 first, since the project now syncs OUTWARD; (4) a named S/4 administrator who can set those up and re-activate them when they expire</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Re-baseline the plan / reduce MVP screen scope / add UI capacity</t>
+          <t>Provide all four, or confirm the connector is deferred</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Overall plan credibility</t>
+          <t>Project sync (D-17), all S/4 mirrors</t>
         </is>
       </c>
       <c r="F17" s="11" t="inlineStr">
@@ -4323,34 +5063,34 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Before committing a client date</t>
+          <t>Before the S/4 connector - NOT blocking upload/download or approvals</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Q-11</t>
+          <t>Q-10</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>UI5 production delivery: how is the app served in Cloud Foundry?</t>
+          <t>Scope re-baseline: personalization + attachments + approvals on every screen</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>mta.yaml has no approuter and no UI module today, and the app bootstraps from a local runtime path</t>
+          <t>Wireframe v12 is 41 modules / 434 screens. The 22-week MVP plan with 1 UI5 developer does not carry this</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Approuter + HTML5 repo (standard) / other</t>
+          <t>Re-baseline the plan / reduce MVP screen scope / add UI capacity</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>Overall plan credibility</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -4360,42 +5100,79 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Before first CF deploy</t>
+          <t>Before committing a client date</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
+          <t>Q-11</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>UI5 production delivery: how is the app served in Cloud Foundry?</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>mta.yaml has no approuter and no UI module today, and the app bootstraps from a local runtime path</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Approuter + HTML5 repo (standard) / other</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Before first CF deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
           <t>Q-12</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>CI/CD tooling</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Prerequisite 4 in the phase plan, still undecided</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>SAP CI/CD service / GitHub Actions / Azure DevOps</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>Before team scales up</t>
         </is>
@@ -4850,7 +5627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5730,27 +6507,27 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>S-24</t>
+          <t>S-35</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Attachments</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Attachment content is stored in the database</t>
+          <t>Four-class budget roll-up blocked on OPEN-01/OPEN-02</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>LargeBinary in HANA is right for the documents that carry legal weight — drawings, permits, signed variations — because they are backed up and restored with the data they belong to. It is the wrong home for thousands of site photographs</t>
+          <t>The spec itself flags that the budget-detail label conflates Class (L1) with control level (L3), and that the six verticals do not map 1:1 onto four classes — SF could be Equipment or Subcontract depending on pool vs vendor-supplied. Every scaffold project's split is wrong until pinned</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Decide whether photo-heavy objects go to an object store instead. It is a per-category switch if decided before volume builds up, and a migration afterwards</t>
+          <t>Answer OPEN-01 and OPEN-02 in the spec; the roll-up is a one-day build once pinned</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
@@ -5767,27 +6544,27 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>S-25</t>
+          <t>S-36</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Attachments</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Nothing scans uploads or limits their size</t>
+          <t>Crew roles have no resource mapping master</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Any authenticated user can upload any file of any size to any object. On a client tenant that is both a malware route and a storage risk</t>
+          <t>Crew composition strings carry role tokens (SK, HLP) that no master resolves to a resource. Unmapped roles fall back to the norm resource, visibly labelled, so demand lands on the wrong resource in plain sight rather than invisibly</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Add a size cap and virus scanning before the first client upload. SAP BTP has a Malware Scanning service; the size cap is configuration</t>
+          <t>Decide where the role-to-resource mapping lives — the Trade Catalogue is the natural home per the wireframe audit</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
@@ -5804,27 +6581,27 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>S-26</t>
+          <t>S-32</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Attachments</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Deleting an attachment breaks the version chain</t>
+          <t>Encumbrance lands in the budget on demand, not on event</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>supersedes points at the previous version. Deleting a middle version leaves the chain dangling, and deleting the document someone approved against destroys the evidence</t>
+          <t>refreshControl sums open reservations into the control record when called. A reservation created after the last refresh is invisible in the budget until someone refreshes</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Block deletion of a superseded version, or of anything attached to a closed approval; mark as obsolete instead</t>
+          <t>Wire the chain to refresh affected budget lines on reservation create/close, or schedule it; on-demand was the honest first cut</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
@@ -5841,35 +6618,405 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
+          <t>S-33</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Spec variance needs a distinct CBS leaf — now ENFORCED as VAL-05</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>The gate fails any CBS leaf carrying two material grades, exactly as spec Part A.3 demands, and budget generation refuses GATE_FAILED while it stands</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Closed by implementation; the stewardship guidance should still cite VAL-05</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>S-34</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Execution</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Reservation encumbrance has no duration dimension</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>estTotal today is unit rate x qty; the seeded canonical thread carried duration-based encumbrances (2 cranes x 320/day x 432 days). Duration needs planning dates the request does not yet carry</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Add period-from/to to request lines when planning dates exist, and price estTotal as qty x rate x days</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>S-30</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Project Setup</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>P6 import matches on project code, so a re-import is refused rather than merged</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Sending a revised P6 file is the normal way a planner works — the schedule changes weekly. Today the second file is rejected as a duplicate code, which is safe but not useful</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Decide what a re-import should mean: refuse, update the header, or reconcile the WBS tree adding and flagging removals. Reconciliation is the one planners will expect and the one that can silently orphan budget lines</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>S-31</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Project Setup</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Only the project header and WBS come across from P6</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Activities, logic, durations, resource assignments and the baseline are all in the file and all ignored. That is the right first cut - KONSTRYX is not a scheduling tool - but it is worth being explicit that P6 remains the schedule of record</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Confirm the boundary: does KONSTRYX ever need activity-level data, or does it stop at WBS?</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>S-27</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Seed data</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>A bad seed row fails silently and looks like an authorization bug</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>The loader cancels the entity's whole change set and logs it at INFO. The symptom is every request returning 403, which sends you looking at the authorization model instead of at a CSV</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Add a startup check that counts loaded rows against the file and fails loudly on a mismatch. Same class of problem as S-05</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>S-28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Project Setup</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Nothing yet stops work against a project that is not in S/4</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>The state is now visible and honest — a project reads NOT_SENT until the connector confirms it — but requisitions, budgets and reservations can still be raised against it. Visibility was the prerequisite; the block is a separate decision</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Decide per document type whether an unsynchronised project blocks creation or only release. Closes the second half of S-17</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>S-29</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Project Setup</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Project numbering is manual</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>A project code is typed in and checked for uniqueness. Number ranges exist and are configurable, and other documents use them, but projects do not — partly because clients often carry an existing code from the contract</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Confirm whether project codes should be issued by a number range, typed, or either depending on the client</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>S-24</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Attachments</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Attachment content is stored in the database</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>LargeBinary in HANA is right for the documents that carry legal weight — drawings, permits, signed variations — because they are backed up and restored with the data they belong to. It is the wrong home for thousands of site photographs</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Decide whether photo-heavy objects go to an object store instead. It is a per-category switch if decided before volume builds up, and a migration afterwards</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>S-25</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Attachments</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Nothing scans uploads or limits their size</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Any authenticated user can upload any file of any size to any object. On a client tenant that is both a malware route and a storage risk</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Add a size cap and virus scanning before the first client upload. SAP BTP has a Malware Scanning service; the size cap is configuration</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>S-26</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Attachments</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Deleting an attachment breaks the version chain</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>supersedes points at the previous version. Deleting a middle version leaves the chain dangling, and deleting the document someone approved against destroys the evidence</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Block deletion of a superseded version, or of anything attached to a closed approval; mark as obsolete instead</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
           <t>S-23</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Frameworks</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>Content packs now carry references</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>Delivered content could previously only hold flat rows, which is why the approval schemes could not ship as content. Packs now resolve a row by natural key at deploy time and match on composite keys</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>Use the same mechanism for the EC&amp;O starter pack (S-13) and for delivered personas</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
+      <c r="F41" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G41" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
@@ -6616,7 +7763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7829,35 +8976,146 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
+          <t>I-33</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Seed data</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>One duplicate key in a seed CSV loads zero rows for that entity, and only logs it at INFO</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>The CSV loader cancels the whole entity's change set on a unique-constraint violation. A duplicated PersonaPermission key therefore loaded no permissions at all and every request returned 403, with nothing at WARN or ERROR explaining why</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Duplicate removed. The behaviour itself is unchanged and will recur — see S-27</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>I-34</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Project Setup</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>@readonly on a projection element does not cover the draft path</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>CAP dispatches a draft edit as DRAFT_PATCH, which the annotation does not gate. The draft displayed syncStatus SENT and an invented S/4 key. Activation stripped them so the stored record was never wrong, but the user was shown something untrue until they saved</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Guarded on the draft event as well as the active one</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>I-32</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Personalization</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Every user could read and write every other user's saved layouts</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>UserVariant was modelled with a user column and no handler behind it, so nothing filtered reads and nothing stopped the payload naming a different owner. A saved filter names projects, counterparties and cost codes, so another person's variant list tells you what they work on</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Owner is taken from the session; reads are narrowed to own plus published; writes to someone else's answer 404 rather than 403 so the key is not confirmed</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
           <t>I-31</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>Approvals</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>withdraw and delegate returned 501 Not Implemented</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>Both actions were declared in CDS without a return type while their handlers set one, which CAP rejects at the protocol layer rather than at build time. Only reachable by calling them - the build was clean</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>Declared returns String on both</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F40" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>

</xml_diff>

<commit_message>
Tracker: regenerate through today's session (risk transfer, distribute-to-WBS, hyperlinks)
79 work items (55 Done / 21 Not started / 2 Blocked / 1 At risk), 22
decisions taken, 12 open decisions still needing you.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Generated from the priced build-up by CBS x cost nature (six); refuses unpriced resources whole; approval via BUD-STD; baseline makes the ledger the only door (PATCH on a baselined amount answers 403); zero-sum paired SHIFT with mandatory reason; refreshControl pulls open reservation encumbrance into the control record</t>
+          <t>Generated from the priced build-up by CBS x cost nature (six); refuses unpriced resources whole; approval via BUD-STD; baseline makes the ledger the only door (PATCH on a baselined amount answers 403); zero-sum paired SHIFT with mandatory reason; refreshControl pulls open reservation encumbrance into the control record; riskTransfer (zero-sum, keyed to a risk reference) and variation (not zero-sum — the one category that moves the budget's own total, keyed to a variation order reference) complete all four KX-BUD-004 categories</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -2090,12 +2090,12 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>25 checks; line amount == sum of its ledger entries asserted per line</t>
+          <t>36 checks; line amount == sum of its ledger entries asserted per line across all four categories; a variation's delta is asserted against the budget's own totalAmount</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>Risk Transfer and Variation documents feeding their ledger categories</t>
+          <t>No standalone Variation Order / Risk register document objects yet — riskTransfer/variation are actions on the budget, referenced by a free-text ID; a formal document with its own approval and number range is a later increment if the business wants one</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2768,7 @@
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>U-07</t>
+          <t>U-10</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -2778,12 +2778,12 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Morning Horizon theme</t>
+          <t>Variant management, adapt filters, table settings and Excel export on the remaining list screens</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
+          <t>Rolled out ListPersonalization (already proven on the RR worklist) to Rate Master, Productivity/Consumption Norms (two independent targets, one screen), Project Templates, and the Promotion Queue. Deliberately NOT applied to Resource Hierarchy or CBS Library — those are TreeTables showing an L1-L5 hierarchy, and generic Sorter/Group panels fight the tree rather than help it; their existing tree-specific search stays. Cost Mapping's exception queue got Export only, no variant management or filter dialog — it is already pre-filtered to "only what needs a decision", so there is nothing left to filter</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -2793,34 +2793,34 @@
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
+          <t>Verified in browser (fresh tab per screen, zero console errors): each table's p13n dialog opens with fields matching its columns exactly, OData row counts intact (Rates 14, Productivity norms 8, Consumption norms 7). Two real bugs found and fixed while wiring this: (1) VariantManagement's showSetAsDefault is not a real property (correct one is supportDefault) — was already wrong on the RR worklist from an earlier session and copied forward before being caught; (2) MasterNorms' two tables collided on duplicate column ids (basis, scope) — XML view ids must be unique across the whole view, not just per control aggregation</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
+          <t>Roll the same treatment to RequestDetail/ChainStep/ResourceDetail if/when those grow list sections; today they are single-object detail pages with nothing to personalize</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>B-01a</t>
+          <t>U-11</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Masters — hybrid scope enforcement</t>
+          <t>Distribute-to-WBS dialog on the Cost Mapping workbench</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
+          <t>UNALLOCATED exception rows had no action — a coordinator could see "0 of 1840 distributed" but had nowhere to act on it. Added a Distribute button opening a dialog over the existing distributeToWBS action: choose TPL-SINGLE (whole line, one element) or TPL-FLOORS/TPL-ZONES (weighted split across several), pick the target WBS element(s), submit. costMappingSummary's exception payload gained boqId (it only carried boqItemId before) so the dialog can address the right BOQ without an extra round trip</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -2830,34 +2830,34 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
+          <t>Verified live end to end for all three templates. TPL-SINGLE: item 1.E.1.1.01 (0 of 1840) onto WBS-0.10. TPL-ZONES: item 1.E.2.2.01 (0 of 682) split 30/70 across WBS-0.10/WBS-1.02, landing at exactly 204.6/477.4 (682.0 to the tenth) with template and splitBasis recorded on the allocation rows. Full regression unaffected throughout: 13 suites / 271 checks green each time</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Two real bugs found and fixed while building this. (1) `class` is not a valid constructor setting in JS-built controls (only in XML) — silently no-ops with a console warning; fixed here and on MasterTemplates' pre-existing instantiate dialog, both now use addStyleClass(). (2) A genuine SAPUI5-vs-CAP encoding mismatch: the v4 ODataModel serialises a Decimal nested inside an array-of-complex-type action parameter (targets: array of WBSTarget) as a JSON string, and CAP's OData V4 deserialiser refuses a quoted decimal on that property ("Invalid value for property 'weight'") — confirmed by direct curl: the identical payload succeeds the moment weight is a bare JSON number, fails identically whether sent as a JS number or a JS string through the typed model API. Worked around by posting distributeToWBS as a raw authenticated fetch instead of the model's typed action-parameter path; template/itemNos still round-trip fine through the model elsewhere since they are not complex-type array members</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>B-01b</t>
+          <t>U-12</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Masters — promotion queue (mdg)</t>
+          <t>Resource hyperlinks on Rate Master and Norms</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
+          <t>The resource/material column on Rate Master and both Norms tables (Productivity, Consumption) was plain text — no way to jump to the resource's master record from a rate or a norm. Wired the existing ObjectLinks "resource" registry (Resource Master / Rate Master / Norms) onto all three columns; no registry changes needed since material is modelled as ResourceNode (same entity resource points to)</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
@@ -2867,34 +2867,34 @@
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
+          <t>Verified in browser (fresh tab, zero console errors) on all three tables: link press opens the popover with all three targets, Resource Master target navigates to #/masters/resource/{code} correctly</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PromotionQueue's objectKey could link to its underlying master too, but objectType there is a free-text label (Resource/CBS/Rate/...), not a typed reference the registry can resolve without new backend support — left alone rather than guessing a mapping</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>B-01c</t>
+          <t>U-07</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Masters — validation rules</t>
+          <t>Morning Horizon theme</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
+          <t>sap_horizon is Morning Horizon; already the bootstrap theme</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -2904,19 +2904,19 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
+          <t>index.html bootstraps data-sap-ui-theme=sap_horizon</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Must be inherited from the shell once launchpad-hosted, never hard-coded</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>B-01d</t>
+          <t>B-01a</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
@@ -2926,12 +2926,12 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Masters — remaining entities catalogued</t>
+          <t>Masters — hybrid scope enforcement</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>CBS library, productivity and consumption norms, templates, material mirror added to the authorization catalogue</t>
+          <t>Reads on any entity carrying the scoped aspect narrow to GROUP or the user's own companies; aspect duck-typed from the model, not a name list</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>CBS library picked up isolation, promotion and L1-L3 depth checks with no CBS-specific code — both handlers duck-type the scoped aspect</t>
+          <t>Two stewards in different legal entities each see 5 group masters + their own local one, and neither sees the other's</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -2953,7 +2953,7 @@
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>B-01e</t>
+          <t>B-01b</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -2963,12 +2963,12 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Masters — list screens</t>
+          <t>Masters — promotion queue (mdg)</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
+          <t>requestPromotion on the master, approve/reject on the queue; scope is never edited directly</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
+          <t>EQ-LOC-INFC invisible to PMI, requested, approved, then visible — reason, decider and outcome recorded</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -2990,7 +2990,7 @@
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>B-01f</t>
+          <t>B-01c</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
@@ -3000,12 +3000,12 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Masters — object page</t>
+          <t>Masters — validation rules</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
+          <t>Level/parent agreement, code uniqueness per scope, rate effective-date clashes, promotion collision check</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
+          <t>Valid L1 accepted; L5 with no parent, L1 given a parent, L3 under an L5, duplicate code and group-vs-local clash all rejected with 409 and a specific message; promotion blocked while INFC and PMI both hold EQ-DUP, naming both</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
@@ -3027,7 +3027,7 @@
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>B-01h</t>
+          <t>B-01d</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -3037,12 +3037,12 @@
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Masters — draft editing</t>
+          <t>Masters — remaining entities catalogued</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
+          <t>CBS library, productivity and consumption norms, templates, material mirror added to the authorization catalogue</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -3052,19 +3052,19 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
+          <t>CBS library picked up isolation, promotion and L1-L3 depth checks with no CBS-specific code — both handlers duck-type the scoped aspect</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>B-01g</t>
+          <t>B-01e</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
@@ -3074,12 +3074,12 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>Masters — productivity and consumption norms</t>
+          <t>Masters — list screens</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>One screen, two tabs; plus a material branch in the resource tree so consumption norms attach to materials rather than equipment</t>
+          <t>Resource hierarchy, CBS library, rate master and promotion queue, all on live OData with server-side filters</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>4 productivity norms with crew composition, 3 consumption norms with wastage; group 105 kg/m3 rebar against INFC's own 112 kg for coastal detailing</t>
+          <t>Verified by screenshot: 7 resources (PMI's local one correctly absent from an INFC session), 7 CBS nodes, 8 rates, 1 pending promotion</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3101,7 +3101,7 @@
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>B-02a</t>
+          <t>B-01f</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
@@ -3111,12 +3111,12 @@
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Templates — model and instantiation</t>
+          <t>Masters — object page</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+          <t>Header facts, attributes, rate history and hierarchy children; route carries the code, not the UUID</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+          <t>EQ-TWC-12T shows all three of its rates together; EQ-TOWER shows parent EQ-CRANE and child EQ-TWC-12T</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
@@ -3138,7 +3138,7 @@
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>B-02b</t>
+          <t>B-01h</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
@@ -3148,12 +3148,12 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Templates — screen</t>
+          <t>Masters — draft editing</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>List plus an instantiate dialog offering the projects the user may see; refusal surfaces the service's own message</t>
+          <t>CAP draft: private copy on edit, stored record untouched until activation, resumes an abandoned draft</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
@@ -3163,19 +3163,19 @@
       </c>
       <c r="F68" s="7" t="inlineStr">
         <is>
-          <t>Driven through the UI: TPL-HIGHRISE into PRJ-002 created 7 CBS nodes and 6 planned resources; a second run raised the refusal</t>
+          <t>Edit that was previously rejected now activates and persists; validation still fires on activation</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Object page for a template still to do</t>
+          <t>Edit is on the resource page only; the other masters reuse the same pattern</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>B-03a</t>
+          <t>B-01g</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
@@ -3185,34 +3185,34 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Masters — productivity and consumption norms</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Project master, WBS, CBS instance; S/4 Enterprise Project mirror</t>
-        </is>
-      </c>
-      <c r="E69" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>One screen, two tabs; plus a material branch in the resource tree so consumption norms attach to materials rather than equipment</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
+          <t>4 productivity norms with crew composition, 3 consumption norms with wastage; group 105 kg/m3 rebar against INFC's own 112 kg for coastal detailing</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G69" s="7" t="inlineStr">
-        <is>
-          <t>Next block; S/4 tenant (Q-09) becomes the blocker for the mirror</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>B-02</t>
+          <t>B-02a</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
@@ -3222,34 +3222,34 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Templates</t>
+          <t>Templates — model and instantiation</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Project templates: CBS tree + default resources</t>
-        </is>
-      </c>
-      <c r="E70" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>Template carries construction type, CBS structure and default resources; instantiate copies them into a project, two-pass so children parent to their new instances</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
+          <t>TPL-HIGHRISE into PRJ-002: 7 CBS nodes (3 roots, 4 correctly parented, all traced to library) and 6 planned resources; second run refused</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr">
-        <is>
-          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>B-03</t>
+          <t>B-02b</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -3259,34 +3259,34 @@
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Project Setup</t>
+          <t>Templates — screen</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="inlineStr">
-        <is>
-          <t>Not started</t>
+          <t>List plus an instantiate dialog offering the projects the user may see; refusal surfaces the service's own message</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Driven through the UI: TPL-HIGHRISE into PRJ-002 created 7 CBS nodes and 6 planned resources; a second run raised the refusal</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>After Templates</t>
+          <t>Object page for a template still to do</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>B-04</t>
+          <t>B-03a</t>
         </is>
       </c>
       <c r="B72" s="7" t="inlineStr">
@@ -3296,12 +3296,12 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>Uploads</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
+          <t>Project master, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
@@ -3316,14 +3316,14 @@
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Highest-risk item in the sequence</t>
+          <t>Next block; S/4 tenant (Q-09) becomes the blocker for the mirror</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>B-05</t>
+          <t>B-02</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -3333,12 +3333,12 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Project Planning</t>
+          <t>Templates</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Activity layer, native entity + P6 adapter</t>
+          <t>Project templates: CBS tree + default resources</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
@@ -3353,14 +3353,14 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>After Uploads</t>
+          <t>After Masters</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>B-06</t>
+          <t>B-03</t>
         </is>
       </c>
       <c r="B74" s="7" t="inlineStr">
@@ -3370,12 +3370,12 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>Budgeting</t>
+          <t>Project Setup</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
+          <t>Project, WBS, CBS instance; S/4 Enterprise Project mirror</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
@@ -3390,14 +3390,14 @@
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>After Planning</t>
+          <t>After Templates</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>B-07</t>
+          <t>B-04</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -3407,12 +3407,12 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Project Execution</t>
+          <t>Uploads</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+          <t>BOQ import, estimate import, versioning with progress carry-forward</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
@@ -3427,14 +3427,14 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>After Budgeting</t>
+          <t>Highest-risk item in the sequence</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>B-08</t>
+          <t>B-05</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
@@ -3444,12 +3444,12 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>Project Commercial</t>
+          <t>Project Planning</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>Client billing, variations, payment certificates</t>
+          <t>Activity layer, native entity + P6 adapter</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -3464,14 +3464,14 @@
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>After Execution</t>
+          <t>After Uploads</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>B-09</t>
+          <t>B-06</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -3481,12 +3481,12 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Plant Department</t>
+          <t>Budgeting</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>Equipment, fleet, scaffolding/formwork</t>
+          <t>Budget from BOQ/CBS, 4-category ledger, approval, baseline, encumbrance</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
@@ -3501,71 +3501,71 @@
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>Last per your sequence</t>
+          <t>After Planning</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>B-07</t>
         </is>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>MTA builds a deployable archive</t>
+          <t>Project Execution</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
-        </is>
-      </c>
-      <c r="E78" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>RR-&gt;CLS chain end to end, material + manpower</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr">
         <is>
-          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>After Budgeting</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>B-08</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>First Cloud Foundry deployment</t>
+          <t>Project Commercial</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
-        </is>
-      </c>
-      <c r="E79" s="9" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+          <t>Client billing, variations, payment certificates</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr">
@@ -3575,79 +3575,190 @@
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+          <t>After Execution</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>B-09</t>
         </is>
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>S/4HANA Public Cloud connector</t>
+          <t>Plant Department</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>S4Connection (credentials, CSRF handshake) + S4ProjectConnector (project + WBS push to API_ENTERPRISE_PROJECT_SRV) built and run live against my401381: KX-S4-001 created via release -&gt; sync, confirmed by independent read-back (profile YP05)</t>
-        </is>
-      </c>
-      <c r="E80" s="8" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Equipment, fleet, scaffolding/formwork</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>D-17 loop ran live on the tenant; see Q-09p</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>Scoped to the project scenario only — procurement, finance and BP mirror connectors are not built; BTP destination replaces S4Connection at deployment</t>
+          <t>Last per your sequence</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
         <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>MTA builds a deployable archive</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Approuter + srv + db-deployer; XSUAA, HANA, Destination resources</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>konstryx_0.1.0.mtar 68.9 MB; 234 HDI artifacts and .hdiconfig verified inside the db-deployer</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>First Cloud Foundry deployment</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Push the archive, bind services, verify the app end to end in the cloud</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="inlineStr">
+        <is>
+          <t>Blocked by I-24: needs a KONSTRYX subaccount and cf login</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>S/4HANA Public Cloud connector</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>S4Connection (credentials, CSRF handshake) + S4ProjectConnector (project + WBS push to API_ENTERPRISE_PROJECT_SRV) built and run live against my401381: KX-S4-001 created via release -&gt; sync, confirmed by independent read-back (profile YP05)</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>D-17 loop ran live on the tenant; see Q-09p</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>Scoped to the project scenario only — procurement, finance and BP mirror connectors are not built; BTP destination replaces S4Connection at deployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="7" t="inlineStr">
+        <is>
           <t>D-03</t>
         </is>
       </c>
-      <c r="B81" s="7" t="inlineStr">
+      <c r="B84" s="7" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C81" s="7" t="inlineStr">
+      <c r="C84" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipeline</t>
         </is>
       </c>
-      <c r="D81" s="7" t="inlineStr">
+      <c r="D84" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="E81" s="7" t="inlineStr">
+      <c r="E84" s="7" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F81" s="7" t="inlineStr">
+      <c r="F84" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G81" s="7" t="inlineStr">
+      <c r="G84" s="7" t="inlineStr">
         <is>
           <t>Decision needed</t>
         </is>
@@ -5006,7 +5117,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Communication user + arrangements SAP_COM_0308/0008 active. The connector ran live: KX-S4-001 created in the tenant from KONSTRYX through release -&gt; sync, confirmed by an independent read (profile YP05). Remaining: WBS element read-back navigation name; the other scenarios (procurement, finance) as their modules need them</t>
+          <t>Communication user + arrangements SAP_COM_0308/0008 active. The connector ran live: KX-S4-001 created in the tenant from KONSTRYX through release -&gt; sync, confirmed by an independent read (profile YP05). WBS element read-back also confirmed: A_EnterpriseProject is keyed by ProjectUUID (a GUID), not the Project string — once read with the correct key, to_EnterpriseProjectElement returns both elements (the auto-created root KX-S4-001 and the pushed KX-S4-001.1 'Enabling works'). Remaining: the other scenarios (procurement, finance) as their modules need them</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -5016,7 +5127,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>S/4 connector - project scenario DONE</t>
+          <t>S/4 connector - project scenario DONE, incl. WBS read-back</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Tracker workbook: your answers to Q-05, Q-06, Q-08 and Q-09
Committing the workbook as it stands on disk so the answers are
versioned. They were transcribed into build_tracker.py in the previous
commit; the script does not read column H back, so the two are kept in
step by hand.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KONSTRYX_Status_Tracker.xlsx
+++ b/KONSTRYX_Status_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ziya\Documents\Claude\Projects\KONSTRYX DEV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D0827A-96BD-4CDA-9855-1A5FF81525AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34013708-E868-4016-AE06-50204F9EBBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="1000">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1589" uniqueCount="1003">
   <si>
     <t>KONSTRYX — Build Status Report</t>
   </si>
@@ -3040,6 +3040,15 @@
   </si>
   <si>
     <t>i can upload from different estimator tool like, candy, RAI, etc., so it should be flexible.</t>
+  </si>
+  <si>
+    <t>Both company and group</t>
+  </si>
+  <si>
+    <t>already shared</t>
+  </si>
+  <si>
+    <t>KONSTRYX_UI5_App ignore this folder</t>
   </si>
 </sst>
 </file>
@@ -6459,7 +6468,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>541</v>
       </c>
@@ -6480,6 +6489,9 @@
       </c>
       <c r="G15" s="5" t="s">
         <v>506</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>1000</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="91.2" x14ac:dyDescent="0.3">
@@ -6505,7 +6517,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="68.400000000000006" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="68.400000000000006" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>552</v>
       </c>
@@ -6527,8 +6539,11 @@
       <c r="G17" s="5" t="s">
         <v>557</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="H17" s="16" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>558</v>
       </c>
@@ -6550,8 +6565,11 @@
       <c r="G18" s="5" t="s">
         <v>563</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="H18" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>564</v>
       </c>
@@ -6574,7 +6592,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>569</v>
       </c>

</xml_diff>